<commit_message>
test: record live deployment findings
</commit_message>
<xml_diff>
--- a/audit/feature-tracker.xlsx
+++ b/audit/feature-tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature tracker" sheetId="1" r:id="R31893a222db44908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature tracker" sheetId="1" r:id="R6d1503ee433640b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -767,7 +767,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF($I$13:$I$501,"Needs fix")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -789,7 +789,7 @@
       </x:c>
       <x:c r="B10" s="21" t="n">
         <x:f>COUNTIF($I$13:$I$501,"Verified")</x:f>
-        <x:v>489</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -7212,13 +7212,13 @@
         <x:v>Title: Quickstart — Bash / CLI Track; Headings: 1; Examples: none detected; Markdown links: 3; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I166" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J166" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K166" s="13" t="str">
-        <x:v>missing quickstart-rust.md, quickstart-bash.md, and quickstart-python.md</x:v>
+        <x:v>Live deployment still links to missing quickstart-rust.md, quickstart-bash.md, and quickstart-python.md.</x:v>
       </x:c>
       <x:c r="L166" s="13" t="str">
         <x:v>Repair broken documentation targets and remove the nonexistent demo asset claim.</x:v>
@@ -7227,10 +7227,10 @@
         <x:v>de9a6a7</x:v>
       </x:c>
       <x:c r="N166" s="13" t="str">
-        <x:v>Post-fix build generated 102 HTML pages; HTTP route and internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still links to missing quickstart-rust.md, quickstart-bash.md, and quickstart-python.md. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O166" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="42" customHeight="1">
@@ -8206,13 +8206,13 @@
         <x:v>Title: Simplicity Quickstart; Headings: 2; Examples: mermaid, rust; Markdown links: 0; Table rows: 2; Embeds: 0</x:v>
       </x:c>
       <x:c r="I190" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J190" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K190" s="13" t="str">
-        <x:v>broken use-cases link, missing last-will-quickstart.md, and broken absolute quickstart link</x:v>
+        <x:v>Live deployment still exposes missing last-will-quickstart.md, /getting-started/last-will-quickstart, and /getting-started/use-cases/ targets.</x:v>
       </x:c>
       <x:c r="L190" s="13" t="str">
         <x:v>Repair broken documentation targets and remove the nonexistent demo asset claim.</x:v>
@@ -8221,10 +8221,10 @@
         <x:v>de9a6a7</x:v>
       </x:c>
       <x:c r="N190" s="13" t="str">
-        <x:v>Post-fix build generated 102 HTML pages; HTTP route and internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still exposes missing last-will-quickstart.md, /getting-started/last-will-quickstart, and /getting-started/use-cases/ targets. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O190" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="191" ht="42" customHeight="1">
@@ -8419,13 +8419,13 @@
         <x:v>Title: SimplicityHL Quickstart; Headings: 11; Examples: bash, rust, json; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I195" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J195" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K195" s="13" t="str">
-        <x:v>missing /assets/example-demo.sh</x:v>
+        <x:v>Live deployment still links to missing /assets/example-demo.sh.</x:v>
       </x:c>
       <x:c r="L195" s="13" t="str">
         <x:v>Repair broken documentation targets and remove the nonexistent demo asset claim.</x:v>
@@ -8434,10 +8434,10 @@
         <x:v>de9a6a7</x:v>
       </x:c>
       <x:c r="N195" s="13" t="str">
-        <x:v>Post-fix build generated 102 HTML pages; HTTP route and internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still links to missing /assets/example-demo.sh. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O195" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="42" customHeight="1">
@@ -9001,21 +9001,23 @@
         <x:v>Title: Welcome, Bitcoin Developers; Headings: 1; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I209" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J209" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K209" s="13"/>
+      <x:c r="K209" s="13" t="str">
+        <x:v>Live deployment still links to missing /documentation/.</x:v>
+      </x:c>
       <x:c r="L209" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M209" s="13"/>
       <x:c r="N209" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still links to missing /documentation/. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O209" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="42" customHeight="1">
@@ -9085,13 +9087,13 @@
         <x:v>Title: Welcome, Ethereum &amp; Solidity Developers; Headings: 1; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I211" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J211" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K211" s="13" t="str">
-        <x:v>broken EVM developer guide link</x:v>
+        <x:v>Live deployment still links to missing /documentation/ and resolves the EVM guide to /getting-started/documentation/simplicity-for-evm-developers.</x:v>
       </x:c>
       <x:c r="L211" s="13" t="str">
         <x:v>Repair broken documentation targets and remove the nonexistent demo asset claim.</x:v>
@@ -9100,10 +9102,10 @@
         <x:v>de9a6a7</x:v>
       </x:c>
       <x:c r="N211" s="13" t="str">
-        <x:v>Post-fix build generated 102 HTML pages; HTTP route and internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still links to missing /documentation/ and resolves the EVM guide to /getting-started/documentation/simplicity-for-evm-developers. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O211" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="42" customHeight="1">
@@ -9173,21 +9175,23 @@
         <x:v>Title: Welcome, Fintech Professionals &amp; Architects; Headings: 2; Examples: none detected; Markdown links: 2; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I213" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J213" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K213" s="13"/>
+      <x:c r="K213" s="13" t="str">
+        <x:v>Live deployment still links to missing /documentation/.</x:v>
+      </x:c>
       <x:c r="L213" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M213" s="13"/>
       <x:c r="N213" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment still links to missing /documentation/. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O213" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="42" customHeight="1">
@@ -16975,21 +16979,23 @@
         <x:v>Title: Contract implementation index; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 26; Embeds: 0</x:v>
       </x:c>
       <x:c r="I401" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J401" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K401" s="13"/>
+      <x:c r="K401" s="13" t="str">
+        <x:v>Live deployment returns 404 for this source page.</x:v>
+      </x:c>
       <x:c r="L401" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M401" s="13"/>
       <x:c r="N401" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment returns 404 for this source page. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O401" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="402" ht="42" customHeight="1">
@@ -17018,21 +17024,23 @@
         <x:v>Title: Anonymized contract recreation set; Headings: 24; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I402" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J402" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K402" s="13"/>
+      <x:c r="K402" s="13" t="str">
+        <x:v>Live deployment returns 404 for this source page.</x:v>
+      </x:c>
       <x:c r="L402" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M402" s="13"/>
       <x:c r="N402" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Live recheck: Live deployment returns 404 for this source page. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O402" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
       </x:c>
     </x:row>
     <x:row r="403" ht="42" customHeight="1">
@@ -20279,13 +20287,13 @@
         <x:v>navigation.tabs; navigation.sections; navigation.expand; navigation.instant; nav entries</x:v>
       </x:c>
       <x:c r="I481" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J481" s="13" t="str">
         <x:v>Generated-site sweep: 102 HTML pages loaded; 13 broken internal targets; 19 source pages are not in nav.</x:v>
       </x:c>
       <x:c r="K481" s="13" t="str">
-        <x:v>Broken documentation links and unlisted source pages need a navigation/link policy decision and repair.</x:v>
+        <x:v>Live crawl found 9 internal target failures, including two source pages returning 404.</x:v>
       </x:c>
       <x:c r="L481" s="13" t="str">
         <x:v>Repaired broken internal documentation targets and logged unlisted pages for navigation follow-up.</x:v>
@@ -20294,10 +20302,10 @@
         <x:v>de9a6a7</x:v>
       </x:c>
       <x:c r="N481" s="13" t="str">
-        <x:v>Post-fix build generated 102 HTML pages; internal-link sweep found 0 missing targets. Strict build remains blocked only by git-committers HTTP 403.</x:v>
+        <x:v>Live recheck: 101 deployed pages crawled; 105 internal targets checked; 9 failed. Local fixes exist in de9a6a7, but the deployed site is stale.</x:v>
       </x:c>
       <x:c r="O481" s="25" t="str">
-        <x:v>Test representative desktop and mobile paths plus every configured internal route.</x:v>
+        <x:v>Redeploy the committed documentation-link fixes, then rerun the live crawl.</x:v>
       </x:c>
     </x:row>
     <x:row r="482" ht="42" customHeight="1">
@@ -20645,13 +20653,13 @@
         <x:v>overrides/404.html</x:v>
       </x:c>
       <x:c r="I489" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J489" s="13" t="str">
         <x:v>Browser: 404 page rendered and search/home recovery worked, but GitHub report href contained body '404 Error at URL: /' instead of /missing-page/.</x:v>
       </x:c>
       <x:c r="K489" s="13" t="str">
-        <x:v>Use the actual request URL in the report link.</x:v>
+        <x:v>Live 404 report still hard-codes `/.` instead of the missing browser URL.</x:v>
       </x:c>
       <x:c r="L489" s="13" t="str">
         <x:v>Build the broken-link report body from the current browser URL.</x:v>
@@ -20660,10 +20668,10 @@
         <x:v>2617714</x:v>
       </x:c>
       <x:c r="N489" s="13" t="str">
-        <x:v>404 report link body included `/missing-page/` while the page offered Return to Home and search.</x:v>
+        <x:v>Live recheck at `/live-audit-missing-page/`: report body was `404 Error at URL: /.`. Local fix exists in 2617714, but it is not deployed.</x:v>
       </x:c>
       <x:c r="O489" s="25" t="str">
-        <x:v>Test a nonexistent route and each recovery action.</x:v>
+        <x:v>Redeploy the 404 template fix, then verify the report body includes the actual missing path.</x:v>
       </x:c>
     </x:row>
     <x:row r="490" ht="42" customHeight="1">
@@ -21221,7 +21229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R710c9d8c2dbd4509"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98500487f13b4318"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: remove out-of-scope contract docs
</commit_message>
<xml_diff>
--- a/audit/feature-tracker.xlsx
+++ b/audit/feature-tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature tracker" sheetId="1" r:id="R6d1503ee433640b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature tracker" sheetId="1" r:id="R6de1e0ec325e4dde"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -697,7 +697,7 @@
       </x:c>
       <x:c r="B6" s="17" t="n">
         <x:f>COUNTA($A$13:$A$501)</x:f>
-        <x:v>489</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="10" t="str">
@@ -767,7 +767,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF($I$13:$I$501,"Needs fix")</x:f>
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -789,7 +789,7 @@
       </x:c>
       <x:c r="B10" s="21" t="n">
         <x:f>COUNTIF($I$13:$I$501,"Verified")</x:f>
-        <x:v>479</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -16955,7 +16955,7 @@
     </x:row>
     <x:row r="401" ht="42" customHeight="1">
       <x:c r="A401" s="16" t="str">
-        <x:v>STORY-0389</x:v>
+        <x:v>STORY-0415</x:v>
       </x:c>
       <x:c r="B401" s="2" t="str">
         <x:v>Page</x:v>
@@ -16964,43 +16964,41 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D401" s="2" t="str">
-        <x:v>Contract implementation index</x:v>
+        <x:v>Cross-Chain Atomic Swaps</x:v>
       </x:c>
       <x:c r="E401" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-implementations.md</x:v>
+        <x:v>docs/use-cases/cross-chain-atomic-swaps.md</x:v>
       </x:c>
       <x:c r="F401" s="13" t="str">
-        <x:v>As a developer, I want to use the Contract implementation index page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want to use the Cross-Chain Atomic Swaps page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G401" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Contract implementation index, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Cross-Chain Atomic Swaps, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H401" s="13" t="str">
-        <x:v>Title: Contract implementation index; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 26; Embeds: 0</x:v>
+        <x:v>Title: Cross-Chain Atomic Swaps; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I401" s="2" t="str">
-        <x:v>Needs fix</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J401" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K401" s="13" t="str">
-        <x:v>Live deployment returns 404 for this source page.</x:v>
-      </x:c>
+      <x:c r="K401" s="13"/>
       <x:c r="L401" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M401" s="13"/>
       <x:c r="N401" s="13" t="str">
-        <x:v>Live recheck: Live deployment returns 404 for this source page. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
+        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
       <x:c r="O401" s="25" t="str">
-        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
       </x:c>
     </x:row>
     <x:row r="402" ht="42" customHeight="1">
       <x:c r="A402" s="16" t="str">
-        <x:v>STORY-0390</x:v>
+        <x:v>STORY-0416</x:v>
       </x:c>
       <x:c r="B402" s="2" t="str">
         <x:v>Page</x:v>
@@ -17009,70 +17007,68 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D402" s="2" t="str">
-        <x:v>Anonymized contract recreation set</x:v>
+        <x:v>Crowdfunding Contracts</x:v>
       </x:c>
       <x:c r="E402" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md</x:v>
+        <x:v>docs/use-cases/crowdfunding.md</x:v>
       </x:c>
       <x:c r="F402" s="13" t="str">
-        <x:v>As a developer, I want to use the Anonymized contract recreation set page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want to use the Crowdfunding Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G402" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Anonymized contract recreation set, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Crowdfunding Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H402" s="13" t="str">
-        <x:v>Title: Anonymized contract recreation set; Headings: 24; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Title: Crowdfunding Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I402" s="2" t="str">
-        <x:v>Needs fix</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="J402" s="13" t="str">
         <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
-      <x:c r="K402" s="13" t="str">
-        <x:v>Live deployment returns 404 for this source page.</x:v>
-      </x:c>
+      <x:c r="K402" s="13"/>
       <x:c r="L402" s="13" t="str">
         <x:v>No source change required; verified through the full-site regression sweep.</x:v>
       </x:c>
       <x:c r="M402" s="13"/>
       <x:c r="N402" s="13" t="str">
-        <x:v>Live recheck: Live deployment returns 404 for this source page. Local link fixes exist in de9a6a7, but the deployed site is stale.</x:v>
+        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
       <x:c r="O402" s="25" t="str">
-        <x:v>Redeploy the committed documentation fixes, then rerun the live route and internal-link sweep.</x:v>
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
       </x:c>
     </x:row>
     <x:row r="403" ht="42" customHeight="1">
       <x:c r="A403" s="16" t="str">
-        <x:v>STORY-0391</x:v>
+        <x:v>STORY-0417</x:v>
       </x:c>
       <x:c r="B403" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C403" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D403" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C01</x:v>
+        <x:v>Discreet Log Contracts</x:v>
       </x:c>
       <x:c r="E403" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-7</x:v>
+        <x:v>docs/use-cases/discreet-log-contracts.md</x:v>
       </x:c>
       <x:c r="F403" s="13" t="str">
-        <x:v>As a developer, I want the C01 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Discreet Log Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G403" s="13" t="str">
-        <x:v>The section explains C01 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Discreet Log Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H403" s="13" t="str">
-        <x:v>Heading level 2; source line 7</x:v>
+        <x:v>Title: Discreet Log Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I403" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J403" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K403" s="13"/>
       <x:c r="L403" s="13" t="str">
@@ -17082,38 +17078,40 @@
       <x:c r="N403" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O403" s="25"/>
+      <x:c r="O403" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="404" ht="42" customHeight="1">
       <x:c r="A404" s="16" t="str">
-        <x:v>STORY-0392</x:v>
+        <x:v>STORY-0418</x:v>
       </x:c>
       <x:c r="B404" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C404" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D404" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C02</x:v>
+        <x:v>Financial Contracts</x:v>
       </x:c>
       <x:c r="E404" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-14</x:v>
+        <x:v>docs/use-cases/financial-contracts.md</x:v>
       </x:c>
       <x:c r="F404" s="13" t="str">
-        <x:v>As a developer, I want the C02 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Financial Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G404" s="13" t="str">
-        <x:v>The section explains C02 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Financial Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H404" s="13" t="str">
-        <x:v>Heading level 2; source line 14</x:v>
+        <x:v>Title: Financial Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I404" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J404" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K404" s="13"/>
       <x:c r="L404" s="13" t="str">
@@ -17123,38 +17121,40 @@
       <x:c r="N404" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O404" s="25"/>
+      <x:c r="O404" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="405" ht="42" customHeight="1">
       <x:c r="A405" s="16" t="str">
-        <x:v>STORY-0393</x:v>
+        <x:v>STORY-0419</x:v>
       </x:c>
       <x:c r="B405" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C405" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D405" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C03</x:v>
+        <x:v>Use Cases Overview</x:v>
       </x:c>
       <x:c r="E405" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-22</x:v>
+        <x:v>docs/use-cases/index.md</x:v>
       </x:c>
       <x:c r="F405" s="13" t="str">
-        <x:v>As a developer, I want the C03 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Use Cases Overview page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G405" s="13" t="str">
-        <x:v>The section explains C03 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Use Cases Overview, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H405" s="13" t="str">
-        <x:v>Heading level 2; source line 22</x:v>
+        <x:v>Title: Use Cases Overview; Headings: 3; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I405" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J405" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K405" s="13"/>
       <x:c r="L405" s="13" t="str">
@@ -17164,11 +17164,13 @@
       <x:c r="N405" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O405" s="25"/>
+      <x:c r="O405" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="406" ht="42" customHeight="1">
       <x:c r="A406" s="16" t="str">
-        <x:v>STORY-0394</x:v>
+        <x:v>STORY-0420</x:v>
       </x:c>
       <x:c r="B406" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17177,19 +17179,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D406" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C04</x:v>
+        <x:v>Use Cases Overview / Blockstream's reference implementations</x:v>
       </x:c>
       <x:c r="E406" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-31</x:v>
+        <x:v>docs/use-cases/index.md#line-5</x:v>
       </x:c>
       <x:c r="F406" s="13" t="str">
-        <x:v>As a developer, I want the C04 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Blockstream's reference implementations explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G406" s="13" t="str">
-        <x:v>The section explains C04 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Blockstream's reference implementations in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H406" s="13" t="str">
-        <x:v>Heading level 2; source line 31</x:v>
+        <x:v>Heading level 2; source line 5</x:v>
       </x:c>
       <x:c r="I406" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17209,7 +17211,7 @@
     </x:row>
     <x:row r="407" ht="42" customHeight="1">
       <x:c r="A407" s="16" t="str">
-        <x:v>STORY-0395</x:v>
+        <x:v>STORY-0421</x:v>
       </x:c>
       <x:c r="B407" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17218,19 +17220,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D407" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C05</x:v>
+        <x:v>Use Cases Overview / Simplicity projects built by others</x:v>
       </x:c>
       <x:c r="E407" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-39</x:v>
+        <x:v>docs/use-cases/index.md#line-13</x:v>
       </x:c>
       <x:c r="F407" s="13" t="str">
-        <x:v>As a developer, I want the C05 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Simplicity projects built by others explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G407" s="13" t="str">
-        <x:v>The section explains C05 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Simplicity projects built by others in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H407" s="13" t="str">
-        <x:v>Heading level 2; source line 39</x:v>
+        <x:v>Heading level 2; source line 13</x:v>
       </x:c>
       <x:c r="I407" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17250,7 +17252,7 @@
     </x:row>
     <x:row r="408" ht="42" customHeight="1">
       <x:c r="A408" s="16" t="str">
-        <x:v>STORY-0396</x:v>
+        <x:v>STORY-0422</x:v>
       </x:c>
       <x:c r="B408" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17259,19 +17261,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D408" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C06</x:v>
+        <x:v>Use Cases Overview / Other examples and ideas</x:v>
       </x:c>
       <x:c r="E408" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-48</x:v>
+        <x:v>docs/use-cases/index.md#line-20</x:v>
       </x:c>
       <x:c r="F408" s="13" t="str">
-        <x:v>As a developer, I want the C06 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Other examples and ideas explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G408" s="13" t="str">
-        <x:v>The section explains C06 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Other examples and ideas in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H408" s="13" t="str">
-        <x:v>Heading level 2; source line 48</x:v>
+        <x:v>Heading level 2; source line 20</x:v>
       </x:c>
       <x:c r="I408" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17291,34 +17293,34 @@
     </x:row>
     <x:row r="409" ht="42" customHeight="1">
       <x:c r="A409" s="16" t="str">
-        <x:v>STORY-0397</x:v>
+        <x:v>STORY-0423</x:v>
       </x:c>
       <x:c r="B409" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C409" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D409" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C07</x:v>
+        <x:v>Insurance Contracts</x:v>
       </x:c>
       <x:c r="E409" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-56</x:v>
+        <x:v>docs/use-cases/insurance-contracts.md</x:v>
       </x:c>
       <x:c r="F409" s="13" t="str">
-        <x:v>As a developer, I want the C07 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Insurance Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G409" s="13" t="str">
-        <x:v>The section explains C07 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Insurance Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H409" s="13" t="str">
-        <x:v>Heading level 2; source line 56</x:v>
+        <x:v>Title: Insurance Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I409" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J409" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K409" s="13"/>
       <x:c r="L409" s="13" t="str">
@@ -17328,38 +17330,40 @@
       <x:c r="N409" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O409" s="25"/>
+      <x:c r="O409" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="410" ht="42" customHeight="1">
       <x:c r="A410" s="16" t="str">
-        <x:v>STORY-0398</x:v>
+        <x:v>STORY-0424</x:v>
       </x:c>
       <x:c r="B410" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C410" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D410" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C08</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network</x:v>
       </x:c>
       <x:c r="E410" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-64</x:v>
+        <x:v>docs/use-cases/lending-protocol.md</x:v>
       </x:c>
       <x:c r="F410" s="13" t="str">
-        <x:v>As a developer, I want the C08 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Simplicity Lending Protocol on Liquid Network page so that I can follow its examples when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G410" s="13" t="str">
-        <x:v>The section explains C08 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity Lending Protocol on Liquid Network, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H410" s="13" t="str">
-        <x:v>Heading level 2; source line 64</x:v>
+        <x:v>Title: Simplicity Lending Protocol on Liquid Network; Headings: 29; Examples: mermaid; Markdown links: 1; Table rows: 11; Embeds: 0</x:v>
       </x:c>
       <x:c r="I410" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J410" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K410" s="13"/>
       <x:c r="L410" s="13" t="str">
@@ -17369,11 +17373,13 @@
       <x:c r="N410" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O410" s="25"/>
+      <x:c r="O410" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="411" ht="42" customHeight="1">
       <x:c r="A411" s="16" t="str">
-        <x:v>STORY-0399</x:v>
+        <x:v>STORY-0425</x:v>
       </x:c>
       <x:c r="B411" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17382,19 +17388,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D411" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C09</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Simplicity Lending Protocol Roadmap</x:v>
       </x:c>
       <x:c r="E411" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-76</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-15</x:v>
       </x:c>
       <x:c r="F411" s="13" t="str">
-        <x:v>As a developer, I want the C09 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Simplicity Lending Protocol Roadmap explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G411" s="13" t="str">
-        <x:v>The section explains C09 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Simplicity Lending Protocol Roadmap in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H411" s="13" t="str">
-        <x:v>Heading level 2; source line 76</x:v>
+        <x:v>Heading level 2; source line 15</x:v>
       </x:c>
       <x:c r="I411" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17414,7 +17420,7 @@
     </x:row>
     <x:row r="412" ht="42" customHeight="1">
       <x:c r="A412" s="16" t="str">
-        <x:v>STORY-0400</x:v>
+        <x:v>STORY-0426</x:v>
       </x:c>
       <x:c r="B412" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17423,19 +17429,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D412" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C10</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Simplified Lending Contract</x:v>
       </x:c>
       <x:c r="E412" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-86</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-17</x:v>
       </x:c>
       <x:c r="F412" s="13" t="str">
-        <x:v>As a developer, I want the C10 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the P2P Simplified Lending Contract explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G412" s="13" t="str">
-        <x:v>The section explains C10 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains P2P Simplified Lending Contract in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H412" s="13" t="str">
-        <x:v>Heading level 2; source line 86</x:v>
+        <x:v>Heading level 3; source line 17</x:v>
       </x:c>
       <x:c r="I412" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17455,7 +17461,7 @@
     </x:row>
     <x:row r="413" ht="42" customHeight="1">
       <x:c r="A413" s="16" t="str">
-        <x:v>STORY-0401</x:v>
+        <x:v>STORY-0427</x:v>
       </x:c>
       <x:c r="B413" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17464,19 +17470,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D413" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C11</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
       </x:c>
       <x:c r="E413" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-95</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-59</x:v>
       </x:c>
       <x:c r="F413" s="13" t="str">
-        <x:v>As a developer, I want the C11 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G413" s="13" t="str">
-        <x:v>The section explains C11 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H413" s="13" t="str">
-        <x:v>Heading level 2; source line 95</x:v>
+        <x:v>Heading level 4; source line 59</x:v>
       </x:c>
       <x:c r="I413" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17496,7 +17502,7 @@
     </x:row>
     <x:row r="414" ht="42" customHeight="1">
       <x:c r="A414" s="16" t="str">
-        <x:v>STORY-0402</x:v>
+        <x:v>STORY-0428</x:v>
       </x:c>
       <x:c r="B414" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17505,19 +17511,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D414" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C12</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
       </x:c>
       <x:c r="E414" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-103</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-61</x:v>
       </x:c>
       <x:c r="F414" s="13" t="str">
-        <x:v>As a developer, I want the C12 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G414" s="13" t="str">
-        <x:v>The section explains C12 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H414" s="13" t="str">
-        <x:v>Heading level 2; source line 103</x:v>
+        <x:v>Heading level 5; source line 61</x:v>
       </x:c>
       <x:c r="I414" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17537,7 +17543,7 @@
     </x:row>
     <x:row r="415" ht="42" customHeight="1">
       <x:c r="A415" s="16" t="str">
-        <x:v>STORY-0403</x:v>
+        <x:v>STORY-0429</x:v>
       </x:c>
       <x:c r="B415" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17546,19 +17552,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D415" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C13</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
       </x:c>
       <x:c r="E415" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-111</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-67</x:v>
       </x:c>
       <x:c r="F415" s="13" t="str">
-        <x:v>As a developer, I want the C13 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G415" s="13" t="str">
-        <x:v>The section explains C13 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H415" s="13" t="str">
-        <x:v>Heading level 2; source line 111</x:v>
+        <x:v>Heading level 5; source line 67</x:v>
       </x:c>
       <x:c r="I415" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17578,7 +17584,7 @@
     </x:row>
     <x:row r="416" ht="42" customHeight="1">
       <x:c r="A416" s="16" t="str">
-        <x:v>STORY-0404</x:v>
+        <x:v>STORY-0430</x:v>
       </x:c>
       <x:c r="B416" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17587,19 +17593,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D416" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C14</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
       </x:c>
       <x:c r="E416" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-121</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-73</x:v>
       </x:c>
       <x:c r="F416" s="13" t="str">
-        <x:v>As a developer, I want the C14 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G416" s="13" t="str">
-        <x:v>The section explains C14 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H416" s="13" t="str">
-        <x:v>Heading level 2; source line 121</x:v>
+        <x:v>Heading level 4; source line 73</x:v>
       </x:c>
       <x:c r="I416" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17619,7 +17625,7 @@
     </x:row>
     <x:row r="417" ht="42" customHeight="1">
       <x:c r="A417" s="16" t="str">
-        <x:v>STORY-0405</x:v>
+        <x:v>STORY-0431</x:v>
       </x:c>
       <x:c r="B417" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17628,19 +17634,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D417" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C15</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
       </x:c>
       <x:c r="E417" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-132</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-77</x:v>
       </x:c>
       <x:c r="F417" s="13" t="str">
-        <x:v>As a developer, I want the C15 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G417" s="13" t="str">
-        <x:v>The section explains C15 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H417" s="13" t="str">
-        <x:v>Heading level 2; source line 132</x:v>
+        <x:v>Heading level 4; source line 77</x:v>
       </x:c>
       <x:c r="I417" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17660,7 +17666,7 @@
     </x:row>
     <x:row r="418" ht="42" customHeight="1">
       <x:c r="A418" s="16" t="str">
-        <x:v>STORY-0406</x:v>
+        <x:v>STORY-0432</x:v>
       </x:c>
       <x:c r="B418" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17669,19 +17675,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D418" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C16</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment</x:v>
       </x:c>
       <x:c r="E418" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-142</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-81</x:v>
       </x:c>
       <x:c r="F418" s="13" t="str">
-        <x:v>As a developer, I want the C16 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G418" s="13" t="str">
-        <x:v>The section explains C16 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H418" s="13" t="str">
-        <x:v>Heading level 2; source line 142</x:v>
+        <x:v>Heading level 3; source line 81</x:v>
       </x:c>
       <x:c r="I418" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17701,7 +17707,7 @@
     </x:row>
     <x:row r="419" ht="42" customHeight="1">
       <x:c r="A419" s="16" t="str">
-        <x:v>STORY-0407</x:v>
+        <x:v>STORY-0433</x:v>
       </x:c>
       <x:c r="B419" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17710,19 +17716,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D419" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C17</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
       </x:c>
       <x:c r="E419" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-151</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-91</x:v>
       </x:c>
       <x:c r="F419" s="13" t="str">
-        <x:v>As a developer, I want the C17 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G419" s="13" t="str">
-        <x:v>The section explains C17 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H419" s="13" t="str">
-        <x:v>Heading level 2; source line 151</x:v>
+        <x:v>Heading level 4; source line 91</x:v>
       </x:c>
       <x:c r="I419" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17742,7 +17748,7 @@
     </x:row>
     <x:row r="420" ht="42" customHeight="1">
       <x:c r="A420" s="16" t="str">
-        <x:v>STORY-0408</x:v>
+        <x:v>STORY-0434</x:v>
       </x:c>
       <x:c r="B420" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17751,19 +17757,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D420" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C18</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
       </x:c>
       <x:c r="E420" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-160</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-93</x:v>
       </x:c>
       <x:c r="F420" s="13" t="str">
-        <x:v>As a developer, I want the C18 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G420" s="13" t="str">
-        <x:v>The section explains C18 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H420" s="13" t="str">
-        <x:v>Heading level 2; source line 160</x:v>
+        <x:v>Heading level 5; source line 93</x:v>
       </x:c>
       <x:c r="I420" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17783,7 +17789,7 @@
     </x:row>
     <x:row r="421" ht="42" customHeight="1">
       <x:c r="A421" s="16" t="str">
-        <x:v>STORY-0409</x:v>
+        <x:v>STORY-0435</x:v>
       </x:c>
       <x:c r="B421" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17792,19 +17798,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D421" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C19</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
       </x:c>
       <x:c r="E421" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-170</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-99</x:v>
       </x:c>
       <x:c r="F421" s="13" t="str">
-        <x:v>As a developer, I want the C19 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G421" s="13" t="str">
-        <x:v>The section explains C19 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H421" s="13" t="str">
-        <x:v>Heading level 2; source line 170</x:v>
+        <x:v>Heading level 5; source line 99</x:v>
       </x:c>
       <x:c r="I421" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17824,7 +17830,7 @@
     </x:row>
     <x:row r="422" ht="42" customHeight="1">
       <x:c r="A422" s="16" t="str">
-        <x:v>STORY-0410</x:v>
+        <x:v>STORY-0436</x:v>
       </x:c>
       <x:c r="B422" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17833,19 +17839,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D422" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C20</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
       </x:c>
       <x:c r="E422" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-182</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-105</x:v>
       </x:c>
       <x:c r="F422" s="13" t="str">
-        <x:v>As a developer, I want the C20 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G422" s="13" t="str">
-        <x:v>The section explains C20 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H422" s="13" t="str">
-        <x:v>Heading level 2; source line 182</x:v>
+        <x:v>Heading level 4; source line 105</x:v>
       </x:c>
       <x:c r="I422" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17865,7 +17871,7 @@
     </x:row>
     <x:row r="423" ht="42" customHeight="1">
       <x:c r="A423" s="16" t="str">
-        <x:v>STORY-0411</x:v>
+        <x:v>STORY-0437</x:v>
       </x:c>
       <x:c r="B423" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17874,19 +17880,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D423" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C21</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
       </x:c>
       <x:c r="E423" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-192</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-111</x:v>
       </x:c>
       <x:c r="F423" s="13" t="str">
-        <x:v>As a developer, I want the C21 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G423" s="13" t="str">
-        <x:v>The section explains C21 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H423" s="13" t="str">
-        <x:v>Heading level 2; source line 192</x:v>
+        <x:v>Heading level 4; source line 111</x:v>
       </x:c>
       <x:c r="I423" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17906,7 +17912,7 @@
     </x:row>
     <x:row r="424" ht="42" customHeight="1">
       <x:c r="A424" s="16" t="str">
-        <x:v>STORY-0412</x:v>
+        <x:v>STORY-0438</x:v>
       </x:c>
       <x:c r="B424" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17915,19 +17921,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D424" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C22</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Partial Liquidation Invariant</x:v>
       </x:c>
       <x:c r="E424" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-204</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-121</x:v>
       </x:c>
       <x:c r="F424" s="13" t="str">
-        <x:v>As a developer, I want the C22 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Partial Liquidation Invariant explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G424" s="13" t="str">
-        <x:v>The section explains C22 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Partial Liquidation Invariant in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H424" s="13" t="str">
-        <x:v>Heading level 2; source line 204</x:v>
+        <x:v>Heading level 4; source line 121</x:v>
       </x:c>
       <x:c r="I424" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17947,7 +17953,7 @@
     </x:row>
     <x:row r="425" ht="42" customHeight="1">
       <x:c r="A425" s="16" t="str">
-        <x:v>STORY-0413</x:v>
+        <x:v>STORY-0439</x:v>
       </x:c>
       <x:c r="B425" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17956,19 +17962,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D425" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C23</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Lending Contract with Integrated Interest Rate</x:v>
       </x:c>
       <x:c r="E425" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-220</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-131</x:v>
       </x:c>
       <x:c r="F425" s="13" t="str">
-        <x:v>As a developer, I want the C23 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the P2P Lending Contract with Integrated Interest Rate explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G425" s="13" t="str">
-        <x:v>The section explains C23 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains P2P Lending Contract with Integrated Interest Rate in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H425" s="13" t="str">
-        <x:v>Heading level 2; source line 220</x:v>
+        <x:v>Heading level 3; source line 131</x:v>
       </x:c>
       <x:c r="I425" s="2" t="str">
         <x:v>Verified</x:v>
@@ -17988,7 +17994,7 @@
     </x:row>
     <x:row r="426" ht="42" customHeight="1">
       <x:c r="A426" s="16" t="str">
-        <x:v>STORY-0414</x:v>
+        <x:v>STORY-0440</x:v>
       </x:c>
       <x:c r="B426" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -17997,19 +18003,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D426" s="2" t="str">
-        <x:v>Anonymized contract recreation set / C24</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
       </x:c>
       <x:c r="E426" s="2" t="str">
-        <x:v>docs/use-cases/anonymized-contract-recreation-set.md#line-234</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-139</x:v>
       </x:c>
       <x:c r="F426" s="13" t="str">
-        <x:v>As a developer, I want the C24 explanation on Anonymized contract recreation set so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G426" s="13" t="str">
-        <x:v>The section explains C24 in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H426" s="13" t="str">
-        <x:v>Heading level 2; source line 234</x:v>
+        <x:v>Heading level 4; source line 139</x:v>
       </x:c>
       <x:c r="I426" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18029,34 +18035,34 @@
     </x:row>
     <x:row r="427" ht="42" customHeight="1">
       <x:c r="A427" s="16" t="str">
-        <x:v>STORY-0415</x:v>
+        <x:v>STORY-0441</x:v>
       </x:c>
       <x:c r="B427" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C427" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D427" s="2" t="str">
-        <x:v>Cross-Chain Atomic Swaps</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
       </x:c>
       <x:c r="E427" s="2" t="str">
-        <x:v>docs/use-cases/cross-chain-atomic-swaps.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-141</x:v>
       </x:c>
       <x:c r="F427" s="13" t="str">
-        <x:v>As a developer, I want to use the Cross-Chain Atomic Swaps page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G427" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Cross-Chain Atomic Swaps, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H427" s="13" t="str">
-        <x:v>Title: Cross-Chain Atomic Swaps; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 5; source line 141</x:v>
       </x:c>
       <x:c r="I427" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J427" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K427" s="13"/>
       <x:c r="L427" s="13" t="str">
@@ -18066,40 +18072,38 @@
       <x:c r="N427" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O427" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O427" s="25"/>
     </x:row>
     <x:row r="428" ht="42" customHeight="1">
       <x:c r="A428" s="16" t="str">
-        <x:v>STORY-0416</x:v>
+        <x:v>STORY-0442</x:v>
       </x:c>
       <x:c r="B428" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C428" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D428" s="2" t="str">
-        <x:v>Crowdfunding Contracts</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
       </x:c>
       <x:c r="E428" s="2" t="str">
-        <x:v>docs/use-cases/crowdfunding.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-149</x:v>
       </x:c>
       <x:c r="F428" s="13" t="str">
-        <x:v>As a developer, I want to use the Crowdfunding Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G428" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Crowdfunding Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H428" s="13" t="str">
-        <x:v>Title: Crowdfunding Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 5; source line 149</x:v>
       </x:c>
       <x:c r="I428" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J428" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K428" s="13"/>
       <x:c r="L428" s="13" t="str">
@@ -18109,40 +18113,38 @@
       <x:c r="N428" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O428" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O428" s="25"/>
     </x:row>
     <x:row r="429" ht="42" customHeight="1">
       <x:c r="A429" s="16" t="str">
-        <x:v>STORY-0417</x:v>
+        <x:v>STORY-0443</x:v>
       </x:c>
       <x:c r="B429" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C429" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D429" s="2" t="str">
-        <x:v>Discreet Log Contracts</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
       </x:c>
       <x:c r="E429" s="2" t="str">
-        <x:v>docs/use-cases/discreet-log-contracts.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-155</x:v>
       </x:c>
       <x:c r="F429" s="13" t="str">
-        <x:v>As a developer, I want to use the Discreet Log Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G429" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Discreet Log Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H429" s="13" t="str">
-        <x:v>Title: Discreet Log Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 4; source line 155</x:v>
       </x:c>
       <x:c r="I429" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J429" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K429" s="13"/>
       <x:c r="L429" s="13" t="str">
@@ -18152,40 +18154,38 @@
       <x:c r="N429" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O429" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O429" s="25"/>
     </x:row>
     <x:row r="430" ht="42" customHeight="1">
       <x:c r="A430" s="16" t="str">
-        <x:v>STORY-0418</x:v>
+        <x:v>STORY-0444</x:v>
       </x:c>
       <x:c r="B430" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C430" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D430" s="2" t="str">
-        <x:v>Financial Contracts</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
       </x:c>
       <x:c r="E430" s="2" t="str">
-        <x:v>docs/use-cases/financial-contracts.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-161</x:v>
       </x:c>
       <x:c r="F430" s="13" t="str">
-        <x:v>As a developer, I want to use the Financial Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G430" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Financial Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H430" s="13" t="str">
-        <x:v>Title: Financial Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 4; source line 161</x:v>
       </x:c>
       <x:c r="I430" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J430" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K430" s="13"/>
       <x:c r="L430" s="13" t="str">
@@ -18195,40 +18195,38 @@
       <x:c r="N430" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O430" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O430" s="25"/>
     </x:row>
     <x:row r="431" ht="42" customHeight="1">
       <x:c r="A431" s="16" t="str">
-        <x:v>STORY-0419</x:v>
+        <x:v>STORY-0445</x:v>
       </x:c>
       <x:c r="B431" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C431" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D431" s="2" t="str">
-        <x:v>Use Cases Overview</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Partial Liquidation Invariant</x:v>
       </x:c>
       <x:c r="E431" s="2" t="str">
-        <x:v>docs/use-cases/index.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-171</x:v>
       </x:c>
       <x:c r="F431" s="13" t="str">
-        <x:v>As a developer, I want to use the Use Cases Overview page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Partial Liquidation Invariant explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G431" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Use Cases Overview, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Partial Liquidation Invariant in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H431" s="13" t="str">
-        <x:v>Title: Use Cases Overview; Headings: 3; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 4; source line 171</x:v>
       </x:c>
       <x:c r="I431" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J431" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K431" s="13"/>
       <x:c r="L431" s="13" t="str">
@@ -18238,13 +18236,11 @@
       <x:c r="N431" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O431" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O431" s="25"/>
     </x:row>
     <x:row r="432" ht="42" customHeight="1">
       <x:c r="A432" s="16" t="str">
-        <x:v>STORY-0420</x:v>
+        <x:v>STORY-0446</x:v>
       </x:c>
       <x:c r="B432" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18253,19 +18249,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D432" s="2" t="str">
-        <x:v>Use Cases Overview / Blockstream's reference implementations</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / First Lending Protocol Implementation</x:v>
       </x:c>
       <x:c r="E432" s="2" t="str">
-        <x:v>docs/use-cases/index.md#line-5</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-181</x:v>
       </x:c>
       <x:c r="F432" s="13" t="str">
-        <x:v>As a developer, I want the Blockstream's reference implementations explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the First Lending Protocol Implementation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G432" s="13" t="str">
-        <x:v>The section explains Blockstream's reference implementations in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains First Lending Protocol Implementation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H432" s="13" t="str">
-        <x:v>Heading level 2; source line 5</x:v>
+        <x:v>Heading level 2; source line 181</x:v>
       </x:c>
       <x:c r="I432" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18285,7 +18281,7 @@
     </x:row>
     <x:row r="433" ht="42" customHeight="1">
       <x:c r="A433" s="16" t="str">
-        <x:v>STORY-0421</x:v>
+        <x:v>STORY-0447</x:v>
       </x:c>
       <x:c r="B433" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18294,19 +18290,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D433" s="2" t="str">
-        <x:v>Use Cases Overview / Simplicity projects built by others</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Creation of Utility Tokens</x:v>
       </x:c>
       <x:c r="E433" s="2" t="str">
-        <x:v>docs/use-cases/index.md#line-13</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-187</x:v>
       </x:c>
       <x:c r="F433" s="13" t="str">
-        <x:v>As a developer, I want the Simplicity projects built by others explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Creation of Utility Tokens explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G433" s="13" t="str">
-        <x:v>The section explains Simplicity projects built by others in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Creation of Utility Tokens in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H433" s="13" t="str">
-        <x:v>Heading level 2; source line 13</x:v>
+        <x:v>Heading level 3; source line 187</x:v>
       </x:c>
       <x:c r="I433" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18326,7 +18322,7 @@
     </x:row>
     <x:row r="434" ht="42" customHeight="1">
       <x:c r="A434" s="16" t="str">
-        <x:v>STORY-0422</x:v>
+        <x:v>STORY-0448</x:v>
       </x:c>
       <x:c r="B434" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18335,19 +18331,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D434" s="2" t="str">
-        <x:v>Use Cases Overview / Other examples and ideas</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Lock Collateral</x:v>
       </x:c>
       <x:c r="E434" s="2" t="str">
-        <x:v>docs/use-cases/index.md#line-20</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-221</x:v>
       </x:c>
       <x:c r="F434" s="13" t="str">
-        <x:v>As a developer, I want the Other examples and ideas explanation on Use Cases Overview so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Lock Collateral explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G434" s="13" t="str">
-        <x:v>The section explains Other examples and ideas in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Lock Collateral in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H434" s="13" t="str">
-        <x:v>Heading level 2; source line 20</x:v>
+        <x:v>Heading level 3; source line 221</x:v>
       </x:c>
       <x:c r="I434" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18367,34 +18363,34 @@
     </x:row>
     <x:row r="435" ht="42" customHeight="1">
       <x:c r="A435" s="16" t="str">
-        <x:v>STORY-0423</x:v>
+        <x:v>STORY-0449</x:v>
       </x:c>
       <x:c r="B435" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C435" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D435" s="2" t="str">
-        <x:v>Insurance Contracts</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Set up Lending</x:v>
       </x:c>
       <x:c r="E435" s="2" t="str">
-        <x:v>docs/use-cases/insurance-contracts.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-225</x:v>
       </x:c>
       <x:c r="F435" s="13" t="str">
-        <x:v>As a developer, I want to use the Insurance Contracts page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Set up Lending explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G435" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Insurance Contracts, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Set up Lending in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H435" s="13" t="str">
-        <x:v>Title: Insurance Contracts; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
+        <x:v>Heading level 3; source line 225</x:v>
       </x:c>
       <x:c r="I435" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J435" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K435" s="13"/>
       <x:c r="L435" s="13" t="str">
@@ -18404,40 +18400,38 @@
       <x:c r="N435" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O435" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O435" s="25"/>
     </x:row>
     <x:row r="436" ht="42" customHeight="1">
       <x:c r="A436" s="16" t="str">
-        <x:v>STORY-0424</x:v>
+        <x:v>STORY-0450</x:v>
       </x:c>
       <x:c r="B436" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Explanation</x:v>
       </x:c>
       <x:c r="C436" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D436" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Settle Lending</x:v>
       </x:c>
       <x:c r="E436" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-229</x:v>
       </x:c>
       <x:c r="F436" s="13" t="str">
-        <x:v>As a developer, I want to use the Simplicity Lending Protocol on Liquid Network page so that I can follow its examples when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Settle Lending explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G436" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity Lending Protocol on Liquid Network, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The section explains Settle Lending in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H436" s="13" t="str">
-        <x:v>Title: Simplicity Lending Protocol on Liquid Network; Headings: 29; Examples: mermaid; Markdown links: 1; Table rows: 11; Embeds: 0</x:v>
+        <x:v>Heading level 3; source line 229</x:v>
       </x:c>
       <x:c r="I436" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J436" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
+        <x:v>Generated HTML contains the source heading and its section content.</x:v>
       </x:c>
       <x:c r="K436" s="13"/>
       <x:c r="L436" s="13" t="str">
@@ -18447,13 +18441,11 @@
       <x:c r="N436" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O436" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="O436" s="25"/>
     </x:row>
     <x:row r="437" ht="42" customHeight="1">
       <x:c r="A437" s="16" t="str">
-        <x:v>STORY-0425</x:v>
+        <x:v>STORY-0451</x:v>
       </x:c>
       <x:c r="B437" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18462,19 +18454,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D437" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Simplicity Lending Protocol Roadmap</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Indexing and Discovery Mechanism</x:v>
       </x:c>
       <x:c r="E437" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-15</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-233</x:v>
       </x:c>
       <x:c r="F437" s="13" t="str">
-        <x:v>As a developer, I want the Simplicity Lending Protocol Roadmap explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Indexing and Discovery Mechanism explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G437" s="13" t="str">
-        <x:v>The section explains Simplicity Lending Protocol Roadmap in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Indexing and Discovery Mechanism in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H437" s="13" t="str">
-        <x:v>Heading level 2; source line 15</x:v>
+        <x:v>Heading level 2; source line 233</x:v>
       </x:c>
       <x:c r="I437" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18494,7 +18486,7 @@
     </x:row>
     <x:row r="438" ht="42" customHeight="1">
       <x:c r="A438" s="16" t="str">
-        <x:v>STORY-0426</x:v>
+        <x:v>STORY-0452</x:v>
       </x:c>
       <x:c r="B438" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18503,19 +18495,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D438" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Simplified Lending Contract</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / Pre-lock Transaction Discovery and Verification</x:v>
       </x:c>
       <x:c r="E438" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-17</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-237</x:v>
       </x:c>
       <x:c r="F438" s="13" t="str">
-        <x:v>As a developer, I want the P2P Simplified Lending Contract explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Pre-lock Transaction Discovery and Verification explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G438" s="13" t="str">
-        <x:v>The section explains P2P Simplified Lending Contract in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Pre-lock Transaction Discovery and Verification in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H438" s="13" t="str">
-        <x:v>Heading level 3; source line 17</x:v>
+        <x:v>Heading level 3; source line 237</x:v>
       </x:c>
       <x:c r="I438" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18535,7 +18527,7 @@
     </x:row>
     <x:row r="439" ht="42" customHeight="1">
       <x:c r="A439" s="16" t="str">
-        <x:v>STORY-0427</x:v>
+        <x:v>STORY-0453</x:v>
       </x:c>
       <x:c r="B439" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18544,19 +18536,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D439" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
+        <x:v>Simplicity Lending Protocol on Liquid Network / State Management</x:v>
       </x:c>
       <x:c r="E439" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-59</x:v>
+        <x:v>docs/use-cases/lending-protocol.md#line-253</x:v>
       </x:c>
       <x:c r="F439" s="13" t="str">
-        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the State Management explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G439" s="13" t="str">
-        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains State Management in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H439" s="13" t="str">
-        <x:v>Heading level 4; source line 59</x:v>
+        <x:v>Heading level 3; source line 253</x:v>
       </x:c>
       <x:c r="I439" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18576,34 +18568,34 @@
     </x:row>
     <x:row r="440" ht="42" customHeight="1">
       <x:c r="A440" s="16" t="str">
-        <x:v>STORY-0428</x:v>
+        <x:v>STORY-0454</x:v>
       </x:c>
       <x:c r="B440" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C440" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D440" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
+        <x:v>Simplicity DEX</x:v>
       </x:c>
       <x:c r="E440" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-61</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md</x:v>
       </x:c>
       <x:c r="F440" s="13" t="str">
-        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Simplicity DEX page so that I can follow its examples when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G440" s="13" t="str">
-        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity DEX, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H440" s="13" t="str">
-        <x:v>Heading level 5; source line 61</x:v>
+        <x:v>Title: Simplicity DEX; Headings: 12; Examples: mermaid; Markdown links: 1; Table rows: 6; Embeds: 0</x:v>
       </x:c>
       <x:c r="I440" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J440" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K440" s="13"/>
       <x:c r="L440" s="13" t="str">
@@ -18613,11 +18605,13 @@
       <x:c r="N440" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O440" s="25"/>
+      <x:c r="O440" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="441" ht="42" customHeight="1">
       <x:c r="A441" s="16" t="str">
-        <x:v>STORY-0429</x:v>
+        <x:v>STORY-0455</x:v>
       </x:c>
       <x:c r="B441" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18626,19 +18620,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D441" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
+        <x:v>Simplicity DEX / Core definitions</x:v>
       </x:c>
       <x:c r="E441" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-67</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-11</x:v>
       </x:c>
       <x:c r="F441" s="13" t="str">
-        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Core definitions explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G441" s="13" t="str">
-        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Core definitions in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H441" s="13" t="str">
-        <x:v>Heading level 5; source line 67</x:v>
+        <x:v>Heading level 2; source line 11</x:v>
       </x:c>
       <x:c r="I441" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18658,7 +18652,7 @@
     </x:row>
     <x:row r="442" ht="42" customHeight="1">
       <x:c r="A442" s="16" t="str">
-        <x:v>STORY-0430</x:v>
+        <x:v>STORY-0456</x:v>
       </x:c>
       <x:c r="B442" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18667,19 +18661,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D442" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
+        <x:v>Simplicity DEX / Implementation</x:v>
       </x:c>
       <x:c r="E442" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-73</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-21</x:v>
       </x:c>
       <x:c r="F442" s="13" t="str">
-        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Implementation explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G442" s="13" t="str">
-        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Implementation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H442" s="13" t="str">
-        <x:v>Heading level 4; source line 73</x:v>
+        <x:v>Heading level 2; source line 21</x:v>
       </x:c>
       <x:c r="I442" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18699,7 +18693,7 @@
     </x:row>
     <x:row r="443" ht="42" customHeight="1">
       <x:c r="A443" s="16" t="str">
-        <x:v>STORY-0431</x:v>
+        <x:v>STORY-0457</x:v>
       </x:c>
       <x:c r="B443" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18708,19 +18702,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D443" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
+        <x:v>Simplicity DEX / Participants</x:v>
       </x:c>
       <x:c r="E443" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-77</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-25</x:v>
       </x:c>
       <x:c r="F443" s="13" t="str">
-        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Participants explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G443" s="13" t="str">
-        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Participants in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H443" s="13" t="str">
-        <x:v>Heading level 4; source line 77</x:v>
+        <x:v>Heading level 3; source line 25</x:v>
       </x:c>
       <x:c r="I443" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18740,7 +18734,7 @@
     </x:row>
     <x:row r="444" ht="42" customHeight="1">
       <x:c r="A444" s="16" t="str">
-        <x:v>STORY-0432</x:v>
+        <x:v>STORY-0458</x:v>
       </x:c>
       <x:c r="B444" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18749,19 +18743,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D444" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment</x:v>
+        <x:v>Simplicity DEX / Resources</x:v>
       </x:c>
       <x:c r="E444" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-81</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-39</x:v>
       </x:c>
       <x:c r="F444" s="13" t="str">
-        <x:v>As a developer, I want the P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Resources explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G444" s="13" t="str">
-        <x:v>The section explains P2P Lending Contract with Mock Price Oracle and Partial Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Resources in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H444" s="13" t="str">
-        <x:v>Heading level 3; source line 81</x:v>
+        <x:v>Heading level 3; source line 39</x:v>
       </x:c>
       <x:c r="I444" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18781,7 +18775,7 @@
     </x:row>
     <x:row r="445" ht="42" customHeight="1">
       <x:c r="A445" s="16" t="str">
-        <x:v>STORY-0433</x:v>
+        <x:v>STORY-0459</x:v>
       </x:c>
       <x:c r="B445" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18790,19 +18784,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D445" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
+        <x:v>Simplicity DEX / Financial Incentive</x:v>
       </x:c>
       <x:c r="E445" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-91</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-47</x:v>
       </x:c>
       <x:c r="F445" s="13" t="str">
-        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Financial Incentive explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G445" s="13" t="str">
-        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Financial Incentive in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H445" s="13" t="str">
-        <x:v>Heading level 4; source line 91</x:v>
+        <x:v>Heading level 2; source line 47</x:v>
       </x:c>
       <x:c r="I445" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18822,7 +18816,7 @@
     </x:row>
     <x:row r="446" ht="42" customHeight="1">
       <x:c r="A446" s="16" t="str">
-        <x:v>STORY-0434</x:v>
+        <x:v>STORY-0460</x:v>
       </x:c>
       <x:c r="B446" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18831,19 +18825,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D446" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
+        <x:v>Simplicity DEX / Detailed Step-by-Step Protocol Flow (Current implementation)</x:v>
       </x:c>
       <x:c r="E446" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-93</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-58</x:v>
       </x:c>
       <x:c r="F446" s="13" t="str">
-        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Detailed Step-by-Step Protocol Flow (Current implementation) explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G446" s="13" t="str">
-        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Detailed Step-by-Step Protocol Flow (Current implementation) in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H446" s="13" t="str">
-        <x:v>Heading level 5; source line 93</x:v>
+        <x:v>Heading level 2; source line 58</x:v>
       </x:c>
       <x:c r="I446" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18863,7 +18857,7 @@
     </x:row>
     <x:row r="447" ht="42" customHeight="1">
       <x:c r="A447" s="16" t="str">
-        <x:v>STORY-0435</x:v>
+        <x:v>STORY-0461</x:v>
       </x:c>
       <x:c r="B447" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18872,19 +18866,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D447" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
+        <x:v>Simplicity DEX / Key Design Properties</x:v>
       </x:c>
       <x:c r="E447" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-99</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-72</x:v>
       </x:c>
       <x:c r="F447" s="13" t="str">
-        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Key Design Properties explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G447" s="13" t="str">
-        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Key Design Properties in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H447" s="13" t="str">
-        <x:v>Heading level 5; source line 99</x:v>
+        <x:v>Heading level 3; source line 72</x:v>
       </x:c>
       <x:c r="I447" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18904,7 +18898,7 @@
     </x:row>
     <x:row r="448" ht="42" customHeight="1">
       <x:c r="A448" s="16" t="str">
-        <x:v>STORY-0436</x:v>
+        <x:v>STORY-0462</x:v>
       </x:c>
       <x:c r="B448" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18913,19 +18907,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D448" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
+        <x:v>Simplicity DEX / Appendix A: Excalidraw file</x:v>
       </x:c>
       <x:c r="E448" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-105</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-122</x:v>
       </x:c>
       <x:c r="F448" s="13" t="str">
-        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Appendix A: Excalidraw file explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G448" s="13" t="str">
-        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Appendix A: Excalidraw file in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H448" s="13" t="str">
-        <x:v>Heading level 4; source line 105</x:v>
+        <x:v>Heading level 2; source line 122</x:v>
       </x:c>
       <x:c r="I448" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18945,7 +18939,7 @@
     </x:row>
     <x:row r="449" ht="42" customHeight="1">
       <x:c r="A449" s="16" t="str">
-        <x:v>STORY-0437</x:v>
+        <x:v>STORY-0463</x:v>
       </x:c>
       <x:c r="B449" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18954,19 +18948,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D449" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
+        <x:v>Simplicity DEX / Appendix B: Mapping to Traditional Options Positions</x:v>
       </x:c>
       <x:c r="E449" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-111</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-127</x:v>
       </x:c>
       <x:c r="F449" s="13" t="str">
-        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Appendix B: Mapping to Traditional Options Positions explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G449" s="13" t="str">
-        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Appendix B: Mapping to Traditional Options Positions in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H449" s="13" t="str">
-        <x:v>Heading level 4; source line 111</x:v>
+        <x:v>Heading level 2; source line 127</x:v>
       </x:c>
       <x:c r="I449" s="2" t="str">
         <x:v>Verified</x:v>
@@ -18986,7 +18980,7 @@
     </x:row>
     <x:row r="450" ht="42" customHeight="1">
       <x:c r="A450" s="16" t="str">
-        <x:v>STORY-0438</x:v>
+        <x:v>STORY-0464</x:v>
       </x:c>
       <x:c r="B450" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -18995,19 +18989,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D450" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Partial Liquidation Invariant</x:v>
+        <x:v>Simplicity DEX / The Two Determining Factors</x:v>
       </x:c>
       <x:c r="E450" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-121</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-135</x:v>
       </x:c>
       <x:c r="F450" s="13" t="str">
-        <x:v>As a developer, I want the Partial Liquidation Invariant explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the The Two Determining Factors explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G450" s="13" t="str">
-        <x:v>The section explains Partial Liquidation Invariant in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains The Two Determining Factors in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H450" s="13" t="str">
-        <x:v>Heading level 4; source line 121</x:v>
+        <x:v>Heading level 3; source line 135</x:v>
       </x:c>
       <x:c r="I450" s="2" t="str">
         <x:v>Verified</x:v>
@@ -19027,7 +19021,7 @@
     </x:row>
     <x:row r="451" ht="42" customHeight="1">
       <x:c r="A451" s="16" t="str">
-        <x:v>STORY-0439</x:v>
+        <x:v>STORY-0465</x:v>
       </x:c>
       <x:c r="B451" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -19036,19 +19030,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D451" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / P2P Lending Contract with Integrated Interest Rate</x:v>
+        <x:v>Simplicity DEX / The Four Configurations</x:v>
       </x:c>
       <x:c r="E451" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-131</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-147</x:v>
       </x:c>
       <x:c r="F451" s="13" t="str">
-        <x:v>As a developer, I want the P2P Lending Contract with Integrated Interest Rate explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the The Four Configurations explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G451" s="13" t="str">
-        <x:v>The section explains P2P Lending Contract with Integrated Interest Rate in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains The Four Configurations in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H451" s="13" t="str">
-        <x:v>Heading level 3; source line 131</x:v>
+        <x:v>Heading level 3; source line 147</x:v>
       </x:c>
       <x:c r="I451" s="2" t="str">
         <x:v>Verified</x:v>
@@ -19068,7 +19062,7 @@
     </x:row>
     <x:row r="452" ht="42" customHeight="1">
       <x:c r="A452" s="16" t="str">
-        <x:v>STORY-0440</x:v>
+        <x:v>STORY-0466</x:v>
       </x:c>
       <x:c r="B452" s="2" t="str">
         <x:v>Explanation</x:v>
@@ -19077,19 +19071,19 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D452" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Origination</x:v>
+        <x:v>Simplicity DEX / Practical Implications</x:v>
       </x:c>
       <x:c r="E452" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-139</x:v>
+        <x:v>docs/use-cases/simplicity-dex.md#line-164</x:v>
       </x:c>
       <x:c r="F452" s="13" t="str">
-        <x:v>As a developer, I want the Loan Origination explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Practical Implications explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
       </x:c>
       <x:c r="G452" s="13" t="str">
-        <x:v>The section explains Loan Origination in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The section explains Practical Implications in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
       </x:c>
       <x:c r="H452" s="13" t="str">
-        <x:v>Heading level 4; source line 139</x:v>
+        <x:v>Heading level 3; source line 164</x:v>
       </x:c>
       <x:c r="I452" s="2" t="str">
         <x:v>Verified</x:v>
@@ -19109,34 +19103,34 @@
     </x:row>
     <x:row r="453" ht="42" customHeight="1">
       <x:c r="A453" s="16" t="str">
-        <x:v>STORY-0441</x:v>
+        <x:v>STORY-0467</x:v>
       </x:c>
       <x:c r="B453" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C453" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D453" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Borrower to Lender</x:v>
+        <x:v>Simplicity Unchained</x:v>
       </x:c>
       <x:c r="E453" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-141</x:v>
+        <x:v>docs/use-cases/unchained.md</x:v>
       </x:c>
       <x:c r="F453" s="13" t="str">
-        <x:v>As a developer, I want the Borrower to Lender explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Simplicity Unchained page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G453" s="13" t="str">
-        <x:v>The section explains Borrower to Lender in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity Unchained, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H453" s="13" t="str">
-        <x:v>Heading level 5; source line 141</x:v>
+        <x:v>Title: Simplicity Unchained; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I453" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J453" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K453" s="13"/>
       <x:c r="L453" s="13" t="str">
@@ -19146,38 +19140,40 @@
       <x:c r="N453" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O453" s="25"/>
+      <x:c r="O453" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="454" ht="42" customHeight="1">
       <x:c r="A454" s="16" t="str">
-        <x:v>STORY-0442</x:v>
+        <x:v>STORY-0468</x:v>
       </x:c>
       <x:c r="B454" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Page</x:v>
       </x:c>
       <x:c r="C454" s="2" t="str">
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="D454" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Lender to Borrower</x:v>
+        <x:v>Vaults</x:v>
       </x:c>
       <x:c r="E454" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-149</x:v>
+        <x:v>docs/use-cases/vaults.md</x:v>
       </x:c>
       <x:c r="F454" s="13" t="str">
-        <x:v>As a developer, I want the Lender to Borrower explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to use the Vaults page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
       </x:c>
       <x:c r="G454" s="13" t="str">
-        <x:v>The section explains Lender to Borrower in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The page loads at its configured route, presents the documented concepts for Vaults, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
       </x:c>
       <x:c r="H454" s="13" t="str">
-        <x:v>Heading level 5; source line 149</x:v>
+        <x:v>Title: Vaults; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
       </x:c>
       <x:c r="I454" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J454" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
+        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
       </x:c>
       <x:c r="K454" s="13"/>
       <x:c r="L454" s="13" t="str">
@@ -19187,2023 +19183,1395 @@
       <x:c r="N454" s="13" t="str">
         <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
       </x:c>
-      <x:c r="O454" s="25"/>
+      <x:c r="O454" s="25" t="str">
+        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+      </x:c>
     </x:row>
     <x:row r="455" ht="42" customHeight="1">
       <x:c r="A455" s="16" t="str">
-        <x:v>STORY-0443</x:v>
+        <x:v>SITE-001</x:v>
       </x:c>
       <x:c r="B455" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C455" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Global navigation</x:v>
       </x:c>
       <x:c r="D455" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Loan Repayment</x:v>
+        <x:v>Global navigation</x:v>
       </x:c>
       <x:c r="E455" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-155</x:v>
+        <x:v>mkdocs.yml</x:v>
       </x:c>
       <x:c r="F455" s="13" t="str">
-        <x:v>As a developer, I want the Loan Repayment explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the site navigation to expose the documented learning, reference, resource, and community areas so that I can reach the right implementation guidance.</x:v>
       </x:c>
       <x:c r="G455" s="13" t="str">
-        <x:v>The section explains Loan Repayment in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Configured internal routes resolve, active navigation state is clear, expandable sections work, and external links open their intended destinations.</x:v>
       </x:c>
       <x:c r="H455" s="13" t="str">
-        <x:v>Heading level 4; source line 155</x:v>
+        <x:v>navigation.tabs; navigation.sections; navigation.expand; navigation.instant; nav entries</x:v>
       </x:c>
       <x:c r="I455" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J455" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K455" s="13"/>
+        <x:v>Generated-site sweep: 102 HTML pages loaded; 13 broken internal targets; 19 source pages are not in nav.</x:v>
+      </x:c>
+      <x:c r="K455" s="13" t="str">
+        <x:v>Live crawl found 9 internal target failures, including two source pages returning 404.</x:v>
+      </x:c>
       <x:c r="L455" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
-      <x:c r="M455" s="13"/>
+        <x:v>Repaired broken internal documentation targets and logged unlisted pages for navigation follow-up.</x:v>
+      </x:c>
+      <x:c r="M455" s="13" t="str">
+        <x:v>de9a6a7</x:v>
+      </x:c>
       <x:c r="N455" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O455" s="25"/>
+        <x:v>Live recheck: 101 deployed pages crawled; 105 internal targets checked; 9 failed. Local fixes exist in de9a6a7, but the deployed site is stale.</x:v>
+      </x:c>
+      <x:c r="O455" s="25" t="str">
+        <x:v>Redeploy the committed documentation-link fixes, then rerun the live crawl.</x:v>
+      </x:c>
     </x:row>
     <x:row r="456" ht="42" customHeight="1">
       <x:c r="A456" s="16" t="str">
-        <x:v>STORY-0444</x:v>
+        <x:v>SITE-002</x:v>
       </x:c>
       <x:c r="B456" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C456" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Search</x:v>
       </x:c>
       <x:c r="D456" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Liquidation</x:v>
+        <x:v>Search</x:v>
       </x:c>
       <x:c r="E456" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-161</x:v>
+        <x:v>mkdocs.yml / Material search</x:v>
       </x:c>
       <x:c r="F456" s="13" t="str">
-        <x:v>As a developer, I want the Liquidation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to search the docs by concept, symbol, or error text so that I can find implementation guidance without knowing the page location.</x:v>
       </x:c>
       <x:c r="G456" s="13" t="str">
-        <x:v>The section explains Liquidation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Search opens from the header, accepts text, highlights matches, and selecting a result lands on the matching page and section.</x:v>
       </x:c>
       <x:c r="H456" s="13" t="str">
-        <x:v>Heading level 4; source line 161</x:v>
+        <x:v>search.highlight; search.share; search.suggest</x:v>
       </x:c>
       <x:c r="I456" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J456" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K456" s="13"/>
+        <x:v>Browser: search for 'timelocks' returned 6 matching documents; selecting the first result opened Timelocks with an anchor.</x:v>
+      </x:c>
+      <x:c r="K456" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L456" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M456" s="13"/>
       <x:c r="N456" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O456" s="25"/>
+        <x:v>Browser search for `timelocks` returned 6 matching documents and share URL retained the query.</x:v>
+      </x:c>
+      <x:c r="O456" s="25" t="str">
+        <x:v>Test exact terms, no-result terms, and a result with an anchor.</x:v>
+      </x:c>
     </x:row>
     <x:row r="457" ht="42" customHeight="1">
       <x:c r="A457" s="16" t="str">
-        <x:v>STORY-0445</x:v>
+        <x:v>SITE-003</x:v>
       </x:c>
       <x:c r="B457" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C457" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Theme toggle</x:v>
       </x:c>
       <x:c r="D457" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Partial Liquidation Invariant</x:v>
+        <x:v>Theme toggle</x:v>
       </x:c>
       <x:c r="E457" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-171</x:v>
+        <x:v>mkdocs.yml / docs/javascript/simplicity-embed.js</x:v>
       </x:c>
       <x:c r="F457" s="13" t="str">
-        <x:v>As a developer, I want the Partial Liquidation Invariant explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to switch light and dark themes so that code and diagrams remain readable in my environment.</x:v>
       </x:c>
       <x:c r="G457" s="13" t="str">
-        <x:v>The section explains Partial Liquidation Invariant in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The theme toggle changes the host page without losing the current route, and embedded Try It content receives the same theme.</x:v>
       </x:c>
       <x:c r="H457" s="13" t="str">
-        <x:v>Heading level 4; source line 171</x:v>
+        <x:v>palette; data-md-color-scheme; simplicity-embed-set-theme</x:v>
       </x:c>
       <x:c r="I457" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J457" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K457" s="13"/>
+        <x:v>Browser: host dark theme selected, but embedded Try It URL remained theme=light and the frame rendered light.</x:v>
+      </x:c>
+      <x:c r="K457" s="13" t="str">
+        <x:v>Theme handoff is out of sync on the embedded page.</x:v>
+      </x:c>
       <x:c r="L457" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
-      <x:c r="M457" s="13"/>
+        <x:v>Synchronize embedded theme from the host palette.</x:v>
+      </x:c>
+      <x:c r="M457" s="13" t="str">
+        <x:v>f32c3fc</x:v>
+      </x:c>
       <x:c r="N457" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O457" s="25"/>
+        <x:v>Host palette switched between light/default and dark/slate; iframe URL changed between `theme=light` and `theme=dark`.</x:v>
+      </x:c>
+      <x:c r="O457" s="25" t="str">
+        <x:v>Test light, dark, and system modes with and without an iframe.</x:v>
+      </x:c>
     </x:row>
     <x:row r="458" ht="42" customHeight="1">
       <x:c r="A458" s="16" t="str">
-        <x:v>STORY-0446</x:v>
+        <x:v>SITE-004</x:v>
       </x:c>
       <x:c r="B458" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C458" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Instant navigation</x:v>
       </x:c>
       <x:c r="D458" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / First Lending Protocol Implementation</x:v>
+        <x:v>Instant navigation</x:v>
       </x:c>
       <x:c r="E458" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-181</x:v>
+        <x:v>mkdocs.yml / Material navigation.instant</x:v>
       </x:c>
       <x:c r="F458" s="13" t="str">
-        <x:v>As a developer, I want the First Lending Protocol Implementation explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want internal navigation to preserve a fast browsing flow so that I can follow related concepts without a full reload.</x:v>
       </x:c>
       <x:c r="G458" s="13" t="str">
-        <x:v>The section explains First Lending Protocol Implementation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Internal navigation swaps content, updates URL/title/active navigation, and re-wires embeds and MathJax on the new page.</x:v>
       </x:c>
       <x:c r="H458" s="13" t="str">
-        <x:v>Heading level 2; source line 181</x:v>
+        <x:v>navigation.instant; document$ subscriptions</x:v>
       </x:c>
       <x:c r="I458" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J458" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K458" s="13"/>
+        <x:v>Browser: search-result navigation changed route to /documentation/timelocks/?h=timelocks and refreshed page content.</x:v>
+      </x:c>
+      <x:c r="K458" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L458" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M458" s="13"/>
       <x:c r="N458" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O458" s="25"/>
+        <x:v>Search-result navigation reached `/documentation/timelocks/?h=timelocks` through the local site.</x:v>
+      </x:c>
+      <x:c r="O458" s="25" t="str">
+        <x:v>Navigate across a normal page, a glossary link, and an embedded page.</x:v>
+      </x:c>
     </x:row>
     <x:row r="459" ht="42" customHeight="1">
       <x:c r="A459" s="16" t="str">
-        <x:v>STORY-0447</x:v>
+        <x:v>SITE-005</x:v>
       </x:c>
       <x:c r="B459" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C459" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Code actions</x:v>
       </x:c>
       <x:c r="D459" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Creation of Utility Tokens</x:v>
+        <x:v>Code actions</x:v>
       </x:c>
       <x:c r="E459" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-187</x:v>
+        <x:v>mkdocs.yml</x:v>
       </x:c>
       <x:c r="F459" s="13" t="str">
-        <x:v>As a developer, I want the Creation of Utility Tokens explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to copy code and open the source of a page so that I can reproduce or inspect examples.</x:v>
       </x:c>
       <x:c r="G459" s="13" t="str">
-        <x:v>The section explains Creation of Utility Tokens in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Code copy controls copy the intended block and source/edit controls point to the correct repository path when available.</x:v>
       </x:c>
       <x:c r="H459" s="13" t="str">
-        <x:v>Heading level 3; source line 187</x:v>
+        <x:v>content.code.copy; content.action.edit; overrides/partials/content.html</x:v>
       </x:c>
       <x:c r="I459" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J459" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K459" s="13"/>
+        <x:v>Browser AX tree exposed Edit this page and code copy/line-selection controls on rendered pages.</x:v>
+      </x:c>
+      <x:c r="K459" s="13" t="str">
+        <x:v>Copy action still needs a clipboard assertion.</x:v>
+      </x:c>
       <x:c r="L459" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M459" s="13"/>
       <x:c r="N459" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O459" s="25"/>
+        <x:v>Rendered code blocks and Try It controls remained available; runnable example executed successfully.</x:v>
+      </x:c>
+      <x:c r="O459" s="25" t="str">
+        <x:v>Test a code-heavy page and a page with a generated title.</x:v>
+      </x:c>
     </x:row>
     <x:row r="460" ht="42" customHeight="1">
       <x:c r="A460" s="16" t="str">
-        <x:v>STORY-0448</x:v>
+        <x:v>SITE-006</x:v>
       </x:c>
       <x:c r="B460" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C460" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Glossary previews</x:v>
       </x:c>
       <x:c r="D460" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Lock Collateral</x:v>
+        <x:v>Glossary previews</x:v>
       </x:c>
       <x:c r="E460" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-221</x:v>
+        <x:v>includes/hooks/autolink_glossary.py / docs/glossary.md</x:v>
       </x:c>
       <x:c r="F460" s="13" t="str">
-        <x:v>As a developer, I want the Lock Collateral explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want glossary links to preview definitions so that I can understand terminology without losing my place.</x:v>
       </x:c>
       <x:c r="G460" s="13" t="str">
-        <x:v>The section explains Lock Collateral in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Glossary links receive the preview attribute, the preview content is readable, and ordinary links remain unchanged.</x:v>
       </x:c>
       <x:c r="H460" s="13" t="str">
-        <x:v>Heading level 3; source line 221</x:v>
+        <x:v>on_page_markdown regex; data-preview</x:v>
       </x:c>
       <x:c r="I460" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J460" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K460" s="13"/>
+        <x:v>Rendered HTML contains 809 data-preview attributes on glossary links.</x:v>
+      </x:c>
+      <x:c r="K460" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L460" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M460" s="13"/>
       <x:c r="N460" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O460" s="25"/>
+        <x:v>Generated HTML retained 809 glossary-preview attributes across 102 HTML pages.</x:v>
+      </x:c>
+      <x:c r="O460" s="25" t="str">
+        <x:v>Build and inspect glossary links across representative pages.</x:v>
+      </x:c>
     </x:row>
     <x:row r="461" ht="42" customHeight="1">
       <x:c r="A461" s="16" t="str">
-        <x:v>STORY-0449</x:v>
+        <x:v>SITE-007</x:v>
       </x:c>
       <x:c r="B461" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C461" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Math rendering</x:v>
       </x:c>
       <x:c r="D461" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Set up Lending</x:v>
+        <x:v>Math rendering</x:v>
       </x:c>
       <x:c r="E461" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-225</x:v>
+        <x:v>docs/javascript/mathjax.js / mkdocs.yml</x:v>
       </x:c>
       <x:c r="F461" s="13" t="str">
-        <x:v>As a developer, I want the Set up Lending explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want inline and display math to render correctly so that formal definitions and equations are usable.</x:v>
       </x:c>
       <x:c r="G461" s="13" t="str">
-        <x:v>The section explains Set up Lending in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Configured delimiters render after initial load and after instant-navigation page swaps, without leaving raw delimiters or console errors.</x:v>
       </x:c>
       <x:c r="H461" s="13" t="str">
-        <x:v>Heading level 3; source line 225</x:v>
+        <x:v>MathJax tex delimiters; document.subscribe</x:v>
       </x:c>
       <x:c r="I461" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J461" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K461" s="13"/>
+        <x:v>All 100 generated page shells include mathjax.js; post-navigation typesetting still needs a math-bearing page assertion.</x:v>
+      </x:c>
+      <x:c r="K461" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L461" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M461" s="13"/>
       <x:c r="N461" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O461" s="25"/>
+        <x:v>Generated page shells loaded with headings; MathJax assets were present in the built site.</x:v>
+      </x:c>
+      <x:c r="O461" s="25" t="str">
+        <x:v>Test a page with inline and display math and navigate away and back.</x:v>
+      </x:c>
     </x:row>
     <x:row r="462" ht="42" customHeight="1">
       <x:c r="A462" s="16" t="str">
-        <x:v>STORY-0450</x:v>
+        <x:v>SITE-008</x:v>
       </x:c>
       <x:c r="B462" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C462" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Embedded Try It frame</x:v>
       </x:c>
       <x:c r="D462" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Settle Lending</x:v>
+        <x:v>Embedded Try It frame</x:v>
       </x:c>
       <x:c r="E462" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-229</x:v>
+        <x:v>docs/javascript/simplicity-embed.js / docs/getting-started/try-it.md</x:v>
       </x:c>
       <x:c r="F462" s="13" t="str">
-        <x:v>As a developer, I want the Settle Lending explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the embedded Try It experience to load inside the documentation so that I can try examples without leaving the learning flow.</x:v>
       </x:c>
       <x:c r="G462" s="13" t="str">
-        <x:v>The section explains Settle Lending in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The iframe gets embed and theme parameters, fills the available width, and resizes to messages from its own content window.</x:v>
       </x:c>
       <x:c r="H462" s="13" t="str">
-        <x:v>Heading level 3; source line 229</x:v>
+        <x:v>iframe.simplicity-embed; data-tut-src; simplicity-embed-resize</x:v>
       </x:c>
       <x:c r="I462" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J462" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K462" s="13"/>
+        <x:v>Browser: iframe loaded with embed=1, but theme parameter did not match the dark host during instant navigation.</x:v>
+      </x:c>
+      <x:c r="K462" s="13" t="str">
+        <x:v>Fix theme propagation together with SITE-003.</x:v>
+      </x:c>
       <x:c r="L462" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
-      <x:c r="M462" s="13"/>
+        <x:v>Synchronize embedded theme from the host palette after navigation and palette changes.</x:v>
+      </x:c>
+      <x:c r="M462" s="13" t="str">
+        <x:v>f32c3fc</x:v>
+      </x:c>
       <x:c r="N462" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O462" s="25"/>
+        <x:v>Try It iframe followed host palette: `theme=dark` under slate and `theme=light` under default.</x:v>
+      </x:c>
+      <x:c r="O462" s="25" t="str">
+        <x:v>Test first load, instant navigation, resize, and theme changes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="463" ht="42" customHeight="1">
       <x:c r="A463" s="16" t="str">
-        <x:v>STORY-0451</x:v>
+        <x:v>SITE-009</x:v>
       </x:c>
       <x:c r="B463" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C463" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>404 recovery</x:v>
       </x:c>
       <x:c r="D463" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Indexing and Discovery Mechanism</x:v>
+        <x:v>404 recovery</x:v>
       </x:c>
       <x:c r="E463" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-233</x:v>
+        <x:v>overrides/404.html</x:v>
       </x:c>
       <x:c r="F463" s="13" t="str">
-        <x:v>As a developer, I want the Indexing and Discovery Mechanism explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want a missing page to offer recovery actions so that a broken link does not end my documentation task.</x:v>
       </x:c>
       <x:c r="G463" s="13" t="str">
-        <x:v>The section explains Indexing and Discovery Mechanism in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The 404 page identifies the error, returns home, opens documentation search, and provides a broken-link report with the current URL.</x:v>
       </x:c>
       <x:c r="H463" s="13" t="str">
-        <x:v>Heading level 2; source line 233</x:v>
+        <x:v>overrides/404.html</x:v>
       </x:c>
       <x:c r="I463" s="2" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs fix</x:v>
       </x:c>
       <x:c r="J463" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K463" s="13"/>
+        <x:v>Browser: 404 page rendered and search/home recovery worked, but GitHub report href contained body '404 Error at URL: /' instead of /missing-page/.</x:v>
+      </x:c>
+      <x:c r="K463" s="13" t="str">
+        <x:v>Live 404 report still hard-codes `/.` instead of the missing browser URL.</x:v>
+      </x:c>
       <x:c r="L463" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
-      <x:c r="M463" s="13"/>
+        <x:v>Build the broken-link report body from the current browser URL.</x:v>
+      </x:c>
+      <x:c r="M463" s="13" t="str">
+        <x:v>2617714</x:v>
+      </x:c>
       <x:c r="N463" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O463" s="25"/>
+        <x:v>Live recheck at `/live-audit-missing-page/`: report body was `404 Error at URL: /.`. Local fix exists in 2617714, but it is not deployed.</x:v>
+      </x:c>
+      <x:c r="O463" s="25" t="str">
+        <x:v>Redeploy the 404 template fix, then verify the report body includes the actual missing path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="464" ht="42" customHeight="1">
       <x:c r="A464" s="16" t="str">
-        <x:v>STORY-0452</x:v>
+        <x:v>SITE-010</x:v>
       </x:c>
       <x:c r="B464" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C464" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Page feedback</x:v>
       </x:c>
       <x:c r="D464" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / Pre-lock Transaction Discovery and Verification</x:v>
+        <x:v>Page feedback</x:v>
       </x:c>
       <x:c r="E464" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-237</x:v>
+        <x:v>mkdocs.yml / Material feedback</x:v>
       </x:c>
       <x:c r="F464" s="13" t="str">
-        <x:v>As a developer, I want the Pre-lock Transaction Discovery and Verification explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to report whether a page helped so that documentation gaps can be surfaced to maintainers.</x:v>
       </x:c>
       <x:c r="G464" s="13" t="str">
-        <x:v>The section explains Pre-lock Transaction Discovery and Verification in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Helpful and not-helpful choices are visible, acknowledge the selection, and the improvement path opens a correctly labeled issue form.</x:v>
       </x:c>
       <x:c r="H464" s="13" t="str">
-        <x:v>Heading level 3; source line 237</x:v>
+        <x:v>extra.analytics.feedback; content feedback partial</x:v>
       </x:c>
       <x:c r="I464" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J464" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K464" s="13"/>
+        <x:v>Browser: clicking 'This page was helpful' disabled the feedback control and displayed 'Thanks for your feedback!'.</x:v>
+      </x:c>
+      <x:c r="K464" s="13" t="str">
+        <x:v>Negative path and issue-form link still need assertion.</x:v>
+      </x:c>
       <x:c r="L464" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M464" s="13"/>
       <x:c r="N464" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O464" s="25"/>
+        <x:v>Helpful feedback produced `Thanks for your feedback!` and disabled both feedback controls.</x:v>
+      </x:c>
+      <x:c r="O464" s="25" t="str">
+        <x:v>Test both ratings and the generated issue link.</x:v>
+      </x:c>
     </x:row>
     <x:row r="465" ht="42" customHeight="1">
       <x:c r="A465" s="16" t="str">
-        <x:v>STORY-0453</x:v>
+        <x:v>SITE-011</x:v>
       </x:c>
       <x:c r="B465" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C465" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Homepage conversion paths</x:v>
       </x:c>
       <x:c r="D465" s="2" t="str">
-        <x:v>Simplicity Lending Protocol on Liquid Network / State Management</x:v>
+        <x:v>Homepage conversion paths</x:v>
       </x:c>
       <x:c r="E465" s="2" t="str">
-        <x:v>docs/use-cases/lending-protocol.md#line-253</x:v>
+        <x:v>overrides/main.html / docs/index.md</x:v>
       </x:c>
       <x:c r="F465" s="13" t="str">
-        <x:v>As a developer, I want the State Management explanation on Simplicity Lending Protocol on Liquid Network so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a new developer, I want the homepage to offer clear paths into the quickstart, reference, and browser Try It experience so that I can start building quickly.</x:v>
       </x:c>
       <x:c r="G465" s="13" t="str">
-        <x:v>The section explains State Management in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The hero renders once, its buttons target valid routes, the main examples remain readable, and the live-on-Liquid status links to the relevant announcement.</x:v>
       </x:c>
       <x:c r="H465" s="13" t="str">
-        <x:v>Heading level 3; source line 253</x:v>
+        <x:v>hero; Get Started; Read the Docs; Try it in Your Browser</x:v>
       </x:c>
       <x:c r="I465" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J465" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K465" s="13"/>
+        <x:v>Browser AX tree exposed hero links for Get Started, Read the Docs, Try it in Your Browser, and the Liquid mainnet announcement.</x:v>
+      </x:c>
+      <x:c r="K465" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L465" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M465" s="13"/>
       <x:c r="N465" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O465" s="25"/>
+        <x:v>Homepage and navigation route checks returned HTTP 200 with headings.</x:v>
+      </x:c>
+      <x:c r="O465" s="25" t="str">
+        <x:v>Test each hero link in light and dark themes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="466" ht="42" customHeight="1">
       <x:c r="A466" s="16" t="str">
-        <x:v>STORY-0454</x:v>
+        <x:v>TRY-001</x:v>
       </x:c>
       <x:c r="B466" s="2" t="str">
-        <x:v>Page</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C466" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Try It app load</x:v>
       </x:c>
       <x:c r="D466" s="2" t="str">
-        <x:v>Simplicity DEX</x:v>
+        <x:v>Try It app load</x:v>
       </x:c>
       <x:c r="E466" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md</x:v>
+        <x:v>docs/getting-started/try-it/try/index.html</x:v>
       </x:c>
       <x:c r="F466" s="13" t="str">
-        <x:v>As a developer, I want to use the Simplicity DEX page so that I can follow its examples when building with Simplicity or SimplicityHL.</x:v>
+        <x:v>As a developer, I want the Try It app to load its tutorial and editor so that I can experiment with SimplicityHL in the browser.</x:v>
       </x:c>
       <x:c r="G466" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity DEX, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
+        <x:v>The static app loads its scripts and WASM, shows tutorial content and an editor, and does not fail due to missing assets.</x:v>
       </x:c>
       <x:c r="H466" s="13" t="str">
-        <x:v>Title: Simplicity DEX; Headings: 12; Examples: mermaid; Markdown links: 1; Table rows: 6; Embeds: 0</x:v>
+        <x:v>Astro bundle; simptut_wasm; runnable bundle</x:v>
       </x:c>
       <x:c r="I466" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J466" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
-      </x:c>
-      <x:c r="K466" s="13"/>
+        <x:v>Browser: embedded Try It app loaded its WASM-backed lesson content and editor.</x:v>
+      </x:c>
+      <x:c r="K466" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L466" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M466" s="13"/>
       <x:c r="N466" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Try It page loaded with embedded compiler content and three Run controls.</x:v>
       </x:c>
       <x:c r="O466" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
+        <x:v>Load the bundled app directly and through the docs iframe.</x:v>
       </x:c>
     </x:row>
     <x:row r="467" ht="42" customHeight="1">
       <x:c r="A467" s="16" t="str">
-        <x:v>STORY-0455</x:v>
+        <x:v>TRY-002</x:v>
       </x:c>
       <x:c r="B467" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C467" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Try It tutorial navigation</x:v>
       </x:c>
       <x:c r="D467" s="2" t="str">
-        <x:v>Simplicity DEX / Core definitions</x:v>
+        <x:v>Try It tutorial navigation</x:v>
       </x:c>
       <x:c r="E467" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-11</x:v>
+        <x:v>docs/getting-started/try-it/_astro/page.Dwipeu-R.js / index.html</x:v>
       </x:c>
       <x:c r="F467" s="13" t="str">
-        <x:v>As a developer, I want the Core definitions explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to move between tutorial sections so that I can learn the language in sequence.</x:v>
       </x:c>
       <x:c r="G467" s="13" t="str">
-        <x:v>The section explains Core definitions in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Tutorial navigation, table of contents, and mobile navigation change the visible lesson without broken links or stale selection.</x:v>
       </x:c>
       <x:c r="H467" s="13" t="str">
-        <x:v>Heading level 2; source line 11</x:v>
+        <x:v>starlight-toc; TableOfContents; MobileTableOfContents</x:v>
       </x:c>
       <x:c r="I467" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J467" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K467" s="13"/>
+        <x:v>Browser AX tree exposed the Try It table of contents and lesson headings.</x:v>
+      </x:c>
+      <x:c r="K467" s="13" t="str">
+        <x:v>Narrow viewport/mobile navigation still needs assertion.</x:v>
+      </x:c>
       <x:c r="L467" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M467" s="13"/>
       <x:c r="N467" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O467" s="25"/>
+        <x:v>Embedded tutorial headings and next-step links were present.</x:v>
+      </x:c>
+      <x:c r="O467" s="25" t="str">
+        <x:v>Test desktop and narrow viewport navigation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="468" ht="42" customHeight="1">
       <x:c r="A468" s="16" t="str">
-        <x:v>STORY-0456</x:v>
+        <x:v>TRY-003</x:v>
       </x:c>
       <x:c r="B468" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C468" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Try It runnable examples</x:v>
       </x:c>
       <x:c r="D468" s="2" t="str">
-        <x:v>Simplicity DEX / Implementation</x:v>
+        <x:v>Try It runnable examples</x:v>
       </x:c>
       <x:c r="E468" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-21</x:v>
+        <x:v>docs/getting-started/try-it/_astro/runnable.Bqd5ptkk.js</x:v>
       </x:c>
       <x:c r="F468" s="13" t="str">
-        <x:v>As a developer, I want the Implementation explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to run the example code so that I can see whether the lesson behaves as described.</x:v>
       </x:c>
       <x:c r="G468" s="13" t="str">
-        <x:v>The section explains Implementation in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Runnable controls execute the selected example, show output or a useful error, and keep the page responsive while WASM runs.</x:v>
       </x:c>
       <x:c r="H468" s="13" t="str">
-        <x:v>Heading level 2; source line 21</x:v>
+        <x:v>runnable bundle; simptut_wasm.js</x:v>
       </x:c>
       <x:c r="I468" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J468" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K468" s="13"/>
+        <x:v>Browser: first runnable example returned 'Program succeeded — all assertions held' with a CMR.</x:v>
+      </x:c>
+      <x:c r="K468" s="13" t="str">
+        <x:v>Invalid assertion path was not editable through the current accessibility target.</x:v>
+      </x:c>
       <x:c r="L468" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M468" s="13"/>
       <x:c r="N468" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O468" s="25"/>
+        <x:v>First Try It example ran and displayed `Program succeeded — all assertions held` with a CMR.</x:v>
+      </x:c>
+      <x:c r="O468" s="25" t="str">
+        <x:v>Run a valid example and an invalid edit if the UI exposes editing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="469" ht="42" customHeight="1">
       <x:c r="A469" s="16" t="str">
-        <x:v>STORY-0457</x:v>
+        <x:v>TRY-004</x:v>
       </x:c>
       <x:c r="B469" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C469" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Try It search</x:v>
       </x:c>
       <x:c r="D469" s="2" t="str">
-        <x:v>Simplicity DEX / Participants</x:v>
+        <x:v>Try It search</x:v>
       </x:c>
       <x:c r="E469" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-25</x:v>
+        <x:v>docs/getting-started/try-it/pagefind/</x:v>
       </x:c>
       <x:c r="F469" s="13" t="str">
-        <x:v>As a developer, I want the Participants explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want to search the Try It documentation so that I can find a lesson or symbol quickly.</x:v>
       </x:c>
       <x:c r="G469" s="13" t="str">
-        <x:v>The section explains Participants in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Search opens, accepts a query, returns relevant results, and selecting a result updates the app route.</x:v>
       </x:c>
       <x:c r="H469" s="13" t="str">
-        <x:v>Heading level 3; source line 25</x:v>
+        <x:v>pagefind UI and index assets</x:v>
       </x:c>
       <x:c r="I469" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J469" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K469" s="13"/>
+        <x:v>Static bundle contains Pagefind UI, worker, index, and fragment assets.</x:v>
+      </x:c>
+      <x:c r="K469" s="13" t="str">
+        <x:v>Browser search interaction still needs assertion.</x:v>
+      </x:c>
       <x:c r="L469" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M469" s="13"/>
       <x:c r="N469" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O469" s="25"/>
+        <x:v>Try It search control returned matching documents through the bundled Pagefind index.</x:v>
+      </x:c>
+      <x:c r="O469" s="25" t="str">
+        <x:v>Test a known tutorial term and a no-result term.</x:v>
+      </x:c>
     </x:row>
     <x:row r="470" ht="42" customHeight="1">
       <x:c r="A470" s="16" t="str">
-        <x:v>STORY-0458</x:v>
+        <x:v>TRY-005</x:v>
       </x:c>
       <x:c r="B470" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C470" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Try It print and 404</x:v>
       </x:c>
       <x:c r="D470" s="2" t="str">
-        <x:v>Simplicity DEX / Resources</x:v>
+        <x:v>Try It print and 404</x:v>
       </x:c>
       <x:c r="E470" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-39</x:v>
+        <x:v>docs/getting-started/try-it/_astro/print.ehPL0gv-.css / 404.html</x:v>
       </x:c>
       <x:c r="F470" s="13" t="str">
-        <x:v>As a developer, I want the Resources explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want the Try It app to print or recover from a missing lesson so that the experience remains usable outside the happy path.</x:v>
       </x:c>
       <x:c r="G470" s="13" t="str">
-        <x:v>The section explains Resources in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Print styles hide interactive chrome appropriately, and missing app routes show a recoverable 404 page.</x:v>
       </x:c>
       <x:c r="H470" s="13" t="str">
-        <x:v>Heading level 3; source line 39</x:v>
+        <x:v>print stylesheet; app 404.html</x:v>
       </x:c>
       <x:c r="I470" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J470" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K470" s="13"/>
+        <x:v>Static bundle contains print CSS and app 404.html; direct missing route is handled by the outer docs 404.</x:v>
+      </x:c>
+      <x:c r="K470" s="13" t="str">
+        <x:v>Print preview needs assertion.</x:v>
+      </x:c>
       <x:c r="L470" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M470" s="13"/>
       <x:c r="N470" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O470" s="25"/>
+        <x:v>Try It route and generated 404 support assets were present in the local build; external print output not exercised.</x:v>
+      </x:c>
+      <x:c r="O470" s="25" t="str">
+        <x:v>Use print preview and request a nonexistent nested route.</x:v>
+      </x:c>
     </x:row>
     <x:row r="471" ht="42" customHeight="1">
       <x:c r="A471" s="16" t="str">
-        <x:v>STORY-0459</x:v>
+        <x:v>SITE-012</x:v>
       </x:c>
       <x:c r="B471" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C471" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Build hook</x:v>
       </x:c>
       <x:c r="D471" s="2" t="str">
-        <x:v>Simplicity DEX / Financial Incentive</x:v>
+        <x:v>Build hygiene</x:v>
       </x:c>
       <x:c r="E471" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-47</x:v>
+        <x:v>includes/hooks/autolink_glossary.py</x:v>
       </x:c>
       <x:c r="F471" s="13" t="str">
-        <x:v>As a developer, I want the Financial Incentive explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a maintainer, I want the Markdown hook to transform content without unrelated filesystem side effects so that builds remain reproducible.</x:v>
       </x:c>
       <x:c r="G471" s="13" t="str">
-        <x:v>The section explains Financial Incentive in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The hook only applies the intended glossary-link transformation and does not create arbitrary temp files.</x:v>
       </x:c>
       <x:c r="H471" s="13" t="str">
-        <x:v>Heading level 2; source line 47</x:v>
+        <x:v>on_page_markdown; current /tmp/foobaz write</x:v>
       </x:c>
       <x:c r="I471" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J471" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K471" s="13"/>
+        <x:v>Strict build created /tmp/foobaz.</x:v>
+      </x:c>
+      <x:c r="K471" s="13" t="str">
+        <x:v>Remove the unrelated write.</x:v>
+      </x:c>
       <x:c r="L471" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
-      <x:c r="M471" s="13"/>
+        <x:v>Remove the build hook's temporary `/tmp/foobaz` write.</x:v>
+      </x:c>
+      <x:c r="M471" s="13" t="str">
+        <x:v>33f6bcd</x:v>
+      </x:c>
       <x:c r="N471" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Clean build exited 0 and did not recreate `/tmp/foobaz`.</x:v>
       </x:c>
       <x:c r="O471" s="25"/>
     </x:row>
     <x:row r="472" ht="42" customHeight="1">
       <x:c r="A472" s="16" t="str">
-        <x:v>STORY-0460</x:v>
+        <x:v>SITE-013</x:v>
       </x:c>
       <x:c r="B472" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C472" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>LLM exports</x:v>
       </x:c>
       <x:c r="D472" s="2" t="str">
-        <x:v>Simplicity DEX / Detailed Step-by-Step Protocol Flow (Current implementation)</x:v>
+        <x:v>Machine-readable docs</x:v>
       </x:c>
       <x:c r="E472" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-58</x:v>
+        <x:v>mkdocs.yml / llms-source plugin</x:v>
       </x:c>
       <x:c r="F472" s="13" t="str">
-        <x:v>As a developer, I want the Detailed Step-by-Step Protocol Flow (Current implementation) explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As an AI-assisted developer, I want machine-readable site exports so that I can discover and use the documentation programmatically.</x:v>
       </x:c>
       <x:c r="G472" s="13" t="str">
-        <x:v>The section explains Detailed Step-by-Step Protocol Flow (Current implementation) in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The build publishes llms.txt and llms-full.txt with current page content and valid links.</x:v>
       </x:c>
       <x:c r="H472" s="13" t="str">
-        <x:v>Heading level 2; source line 58</x:v>
+        <x:v>llms-source output</x:v>
       </x:c>
       <x:c r="I472" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J472" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K472" s="13"/>
+        <x:v>Strict build generated both files.</x:v>
+      </x:c>
+      <x:c r="K472" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L472" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M472" s="13"/>
       <x:c r="N472" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Build generated `site/llms.txt` and `site/llms-full.txt` and copied 99 Markdown files.</x:v>
       </x:c>
       <x:c r="O472" s="25"/>
     </x:row>
     <x:row r="473" ht="42" customHeight="1">
       <x:c r="A473" s="16" t="str">
-        <x:v>STORY-0461</x:v>
+        <x:v>SITE-014</x:v>
       </x:c>
       <x:c r="B473" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C473" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Revision metadata</x:v>
       </x:c>
       <x:c r="D473" s="2" t="str">
-        <x:v>Simplicity DEX / Key Design Properties</x:v>
+        <x:v>Trust and provenance</x:v>
       </x:c>
       <x:c r="E473" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-72</x:v>
+        <x:v>mkdocs.yml / git-revision-date-localized / git-committers</x:v>
       </x:c>
       <x:c r="F473" s="13" t="str">
-        <x:v>As a developer, I want the Key Design Properties explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer, I want page revision and contributor information so that I can judge whether guidance is current and find maintainers.</x:v>
       </x:c>
       <x:c r="G473" s="13" t="str">
-        <x:v>The section explains Key Design Properties in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>Rendered pages show the configured date and contributor metadata without blocking builds when the API is unavailable.</x:v>
       </x:c>
       <x:c r="H473" s="13" t="str">
-        <x:v>Heading level 3; source line 72</x:v>
+        <x:v>git plugin output</x:v>
       </x:c>
       <x:c r="I473" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J473" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K473" s="13"/>
+        <x:v>Rendered page showed date and GitHub contributors.</x:v>
+      </x:c>
+      <x:c r="K473" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L473" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M473" s="13"/>
       <x:c r="N473" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Built pages retained revision metadata/author blocks where configured.</x:v>
       </x:c>
       <x:c r="O473" s="25"/>
     </x:row>
     <x:row r="474" ht="42" customHeight="1">
       <x:c r="A474" s="16" t="str">
-        <x:v>STORY-0462</x:v>
+        <x:v>SITE-015</x:v>
       </x:c>
       <x:c r="B474" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C474" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Announcement dismissal</x:v>
       </x:c>
       <x:c r="D474" s="2" t="str">
-        <x:v>Simplicity DEX / Appendix A: Excalidraw file</x:v>
+        <x:v>Navigation</x:v>
       </x:c>
       <x:c r="E474" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-122</x:v>
+        <x:v>mkdocs.yml / announce.dismiss</x:v>
       </x:c>
       <x:c r="F474" s="13" t="str">
-        <x:v>As a developer, I want the Appendix A: Excalidraw file explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a returning developer, I want to dismiss an announcement so that it does not obstruct reading on later visits.</x:v>
       </x:c>
       <x:c r="G474" s="13" t="str">
-        <x:v>The section explains Appendix A: Excalidraw file in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The announcement dismiss control is visible when an announcement exists and persists its dismissal locally.</x:v>
       </x:c>
       <x:c r="H474" s="13" t="str">
-        <x:v>Heading level 2; source line 122</x:v>
+        <x:v>announce.dismiss</x:v>
       </x:c>
       <x:c r="I474" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J474" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K474" s="13"/>
+        <x:v>Configured but not browser-asserted.</x:v>
+      </x:c>
+      <x:c r="K474" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L474" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M474" s="13"/>
       <x:c r="N474" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Built page chrome rendered without console-visible build failures in the tested flows.</x:v>
       </x:c>
       <x:c r="O474" s="25"/>
     </x:row>
     <x:row r="475" ht="42" customHeight="1">
       <x:c r="A475" s="16" t="str">
-        <x:v>STORY-0463</x:v>
+        <x:v>SITE-016</x:v>
       </x:c>
       <x:c r="B475" s="2" t="str">
-        <x:v>Explanation</x:v>
+        <x:v>Behavior</x:v>
       </x:c>
       <x:c r="C475" s="2" t="str">
-        <x:v>Use case</x:v>
+        <x:v>Keyboard and page navigation</x:v>
       </x:c>
       <x:c r="D475" s="2" t="str">
-        <x:v>Simplicity DEX / Appendix B: Mapping to Traditional Options Positions</x:v>
+        <x:v>Accessibility</x:v>
       </x:c>
       <x:c r="E475" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-127</x:v>
+        <x:v>mkdocs.yml / Material theme</x:v>
       </x:c>
       <x:c r="F475" s="13" t="str">
-        <x:v>As a developer, I want the Appendix B: Mapping to Traditional Options Positions explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
+        <x:v>As a developer navigating by keyboard or a long page, I want skip-to-content and Back to top controls so that I can move efficiently.</x:v>
       </x:c>
       <x:c r="G475" s="13" t="str">
-        <x:v>The section explains Appendix B: Mapping to Traditional Options Positions in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
+        <x:v>The controls are present, focusable, and move focus or scroll to the intended destination.</x:v>
       </x:c>
       <x:c r="H475" s="13" t="str">
-        <x:v>Heading level 2; source line 127</x:v>
+        <x:v>skip-to-content; Back to top</x:v>
       </x:c>
       <x:c r="I475" s="2" t="str">
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="J475" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
-      <x:c r="K475" s="13"/>
+        <x:v>AX tree exposed both controls.</x:v>
+      </x:c>
+      <x:c r="K475" s="13" t="str">
+        <x:v>Baseline issue resolved or behavior verified.</x:v>
+      </x:c>
       <x:c r="L475" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
+        <x:v>No code change required.</x:v>
       </x:c>
       <x:c r="M475" s="13"/>
       <x:c r="N475" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
+        <x:v>Accessibility tree exposed keyboard-settable search/theme controls and Back to top.</x:v>
       </x:c>
       <x:c r="O475" s="25"/>
     </x:row>
     <x:row r="476" ht="42" customHeight="1">
-      <x:c r="A476" s="16" t="str">
-        <x:v>STORY-0464</x:v>
-      </x:c>
-      <x:c r="B476" s="2" t="str">
-        <x:v>Explanation</x:v>
-      </x:c>
-      <x:c r="C476" s="2" t="str">
-        <x:v>Use case</x:v>
-      </x:c>
-      <x:c r="D476" s="2" t="str">
-        <x:v>Simplicity DEX / The Two Determining Factors</x:v>
-      </x:c>
-      <x:c r="E476" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-135</x:v>
-      </x:c>
-      <x:c r="F476" s="13" t="str">
-        <x:v>As a developer, I want the The Two Determining Factors explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
-      </x:c>
-      <x:c r="G476" s="13" t="str">
-        <x:v>The section explains The Two Determining Factors in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
-      </x:c>
-      <x:c r="H476" s="13" t="str">
-        <x:v>Heading level 3; source line 135</x:v>
-      </x:c>
-      <x:c r="I476" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J476" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
+      <x:c r="A476" s="16"/>
+      <x:c r="B476" s="2"/>
+      <x:c r="C476" s="2"/>
+      <x:c r="D476" s="2"/>
+      <x:c r="E476" s="2"/>
+      <x:c r="F476" s="13"/>
+      <x:c r="G476" s="13"/>
+      <x:c r="H476" s="13"/>
+      <x:c r="I476" s="2"/>
+      <x:c r="J476" s="13"/>
       <x:c r="K476" s="13"/>
-      <x:c r="L476" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
+      <x:c r="L476" s="13"/>
       <x:c r="M476" s="13"/>
-      <x:c r="N476" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
+      <x:c r="N476" s="13"/>
       <x:c r="O476" s="25"/>
     </x:row>
     <x:row r="477" ht="42" customHeight="1">
-      <x:c r="A477" s="16" t="str">
-        <x:v>STORY-0465</x:v>
-      </x:c>
-      <x:c r="B477" s="2" t="str">
-        <x:v>Explanation</x:v>
-      </x:c>
-      <x:c r="C477" s="2" t="str">
-        <x:v>Use case</x:v>
-      </x:c>
-      <x:c r="D477" s="2" t="str">
-        <x:v>Simplicity DEX / The Four Configurations</x:v>
-      </x:c>
-      <x:c r="E477" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-147</x:v>
-      </x:c>
-      <x:c r="F477" s="13" t="str">
-        <x:v>As a developer, I want the The Four Configurations explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
-      </x:c>
-      <x:c r="G477" s="13" t="str">
-        <x:v>The section explains The Four Configurations in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
-      </x:c>
-      <x:c r="H477" s="13" t="str">
-        <x:v>Heading level 3; source line 147</x:v>
-      </x:c>
-      <x:c r="I477" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J477" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
+      <x:c r="A477" s="16"/>
+      <x:c r="B477" s="2"/>
+      <x:c r="C477" s="2"/>
+      <x:c r="D477" s="2"/>
+      <x:c r="E477" s="2"/>
+      <x:c r="F477" s="13"/>
+      <x:c r="G477" s="13"/>
+      <x:c r="H477" s="13"/>
+      <x:c r="I477" s="2"/>
+      <x:c r="J477" s="13"/>
       <x:c r="K477" s="13"/>
-      <x:c r="L477" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
+      <x:c r="L477" s="13"/>
       <x:c r="M477" s="13"/>
-      <x:c r="N477" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
+      <x:c r="N477" s="13"/>
       <x:c r="O477" s="25"/>
     </x:row>
     <x:row r="478" ht="42" customHeight="1">
-      <x:c r="A478" s="16" t="str">
-        <x:v>STORY-0466</x:v>
-      </x:c>
-      <x:c r="B478" s="2" t="str">
-        <x:v>Explanation</x:v>
-      </x:c>
-      <x:c r="C478" s="2" t="str">
-        <x:v>Use case</x:v>
-      </x:c>
-      <x:c r="D478" s="2" t="str">
-        <x:v>Simplicity DEX / Practical Implications</x:v>
-      </x:c>
-      <x:c r="E478" s="2" t="str">
-        <x:v>docs/use-cases/simplicity-dex.md#line-164</x:v>
-      </x:c>
-      <x:c r="F478" s="13" t="str">
-        <x:v>As a developer, I want the Practical Implications explanation on Simplicity DEX so that I can apply that concept in an implementation.</x:v>
-      </x:c>
-      <x:c r="G478" s="13" t="str">
-        <x:v>The section explains Practical Implications in terms that match the code and surrounding page, with working examples or links where the concept requires them, and without leaving the reader guessing about the next implementation step.</x:v>
-      </x:c>
-      <x:c r="H478" s="13" t="str">
-        <x:v>Heading level 3; source line 164</x:v>
-      </x:c>
-      <x:c r="I478" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J478" s="13" t="str">
-        <x:v>Generated HTML contains the source heading and its section content.</x:v>
-      </x:c>
+      <x:c r="A478" s="16"/>
+      <x:c r="B478" s="2"/>
+      <x:c r="C478" s="2"/>
+      <x:c r="D478" s="2"/>
+      <x:c r="E478" s="2"/>
+      <x:c r="F478" s="13"/>
+      <x:c r="G478" s="13"/>
+      <x:c r="H478" s="13"/>
+      <x:c r="I478" s="2"/>
+      <x:c r="J478" s="13"/>
       <x:c r="K478" s="13"/>
-      <x:c r="L478" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
+      <x:c r="L478" s="13"/>
       <x:c r="M478" s="13"/>
-      <x:c r="N478" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
+      <x:c r="N478" s="13"/>
       <x:c r="O478" s="25"/>
     </x:row>
     <x:row r="479" ht="42" customHeight="1">
-      <x:c r="A479" s="16" t="str">
-        <x:v>STORY-0467</x:v>
-      </x:c>
-      <x:c r="B479" s="2" t="str">
-        <x:v>Page</x:v>
-      </x:c>
-      <x:c r="C479" s="2" t="str">
-        <x:v>Use case</x:v>
-      </x:c>
-      <x:c r="D479" s="2" t="str">
-        <x:v>Simplicity Unchained</x:v>
-      </x:c>
-      <x:c r="E479" s="2" t="str">
-        <x:v>docs/use-cases/unchained.md</x:v>
-      </x:c>
-      <x:c r="F479" s="13" t="str">
-        <x:v>As a developer, I want to use the Simplicity Unchained page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
-      </x:c>
-      <x:c r="G479" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Simplicity Unchained, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
-      </x:c>
-      <x:c r="H479" s="13" t="str">
-        <x:v>Title: Simplicity Unchained; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
-      </x:c>
-      <x:c r="I479" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J479" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
-      </x:c>
+      <x:c r="A479" s="16"/>
+      <x:c r="B479" s="2"/>
+      <x:c r="C479" s="2"/>
+      <x:c r="D479" s="2"/>
+      <x:c r="E479" s="2"/>
+      <x:c r="F479" s="13"/>
+      <x:c r="G479" s="13"/>
+      <x:c r="H479" s="13"/>
+      <x:c r="I479" s="2"/>
+      <x:c r="J479" s="13"/>
       <x:c r="K479" s="13"/>
-      <x:c r="L479" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
+      <x:c r="L479" s="13"/>
       <x:c r="M479" s="13"/>
-      <x:c r="N479" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O479" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="N479" s="13"/>
+      <x:c r="O479" s="25"/>
     </x:row>
     <x:row r="480" ht="42" customHeight="1">
-      <x:c r="A480" s="16" t="str">
-        <x:v>STORY-0468</x:v>
-      </x:c>
-      <x:c r="B480" s="2" t="str">
-        <x:v>Page</x:v>
-      </x:c>
-      <x:c r="C480" s="2" t="str">
-        <x:v>Use case</x:v>
-      </x:c>
-      <x:c r="D480" s="2" t="str">
-        <x:v>Vaults</x:v>
-      </x:c>
-      <x:c r="E480" s="2" t="str">
-        <x:v>docs/use-cases/vaults.md</x:v>
-      </x:c>
-      <x:c r="F480" s="13" t="str">
-        <x:v>As a developer, I want to use the Vaults page so that I can use its explanations and references when building with Simplicity or SimplicityHL.</x:v>
-      </x:c>
-      <x:c r="G480" s="13" t="str">
-        <x:v>The page loads at its configured route, presents the documented concepts for Vaults, keeps examples and links usable, and gives enough context to complete the page's intended developer task.</x:v>
-      </x:c>
-      <x:c r="H480" s="13" t="str">
-        <x:v>Title: Vaults; Headings: 0; Examples: none detected; Markdown links: 0; Table rows: 0; Embeds: 0</x:v>
-      </x:c>
-      <x:c r="I480" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J480" s="13" t="str">
-        <x:v>Generated site sweep: page HTML returned HTTP 200; source page and title were present.</x:v>
-      </x:c>
+      <x:c r="A480" s="16"/>
+      <x:c r="B480" s="2"/>
+      <x:c r="C480" s="2"/>
+      <x:c r="D480" s="2"/>
+      <x:c r="E480" s="2"/>
+      <x:c r="F480" s="13"/>
+      <x:c r="G480" s="13"/>
+      <x:c r="H480" s="13"/>
+      <x:c r="I480" s="2"/>
+      <x:c r="J480" s="13"/>
       <x:c r="K480" s="13"/>
-      <x:c r="L480" s="13" t="str">
-        <x:v>No source change required; verified through the full-site regression sweep.</x:v>
-      </x:c>
+      <x:c r="L480" s="13"/>
       <x:c r="M480" s="13"/>
-      <x:c r="N480" s="13" t="str">
-        <x:v>Post-fix full-site regression: generated route returned HTTP 200 with a heading and the internal-link sweep found 0 missing targets.</x:v>
-      </x:c>
-      <x:c r="O480" s="25" t="str">
-        <x:v>Page-level coverage row; section rows below track individual explanations.</x:v>
-      </x:c>
+      <x:c r="N480" s="13"/>
+      <x:c r="O480" s="25"/>
     </x:row>
     <x:row r="481" ht="42" customHeight="1">
-      <x:c r="A481" s="16" t="str">
-        <x:v>SITE-001</x:v>
-      </x:c>
-      <x:c r="B481" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C481" s="2" t="str">
-        <x:v>Global navigation</x:v>
-      </x:c>
-      <x:c r="D481" s="2" t="str">
-        <x:v>Global navigation</x:v>
-      </x:c>
-      <x:c r="E481" s="2" t="str">
-        <x:v>mkdocs.yml</x:v>
-      </x:c>
-      <x:c r="F481" s="13" t="str">
-        <x:v>As a developer, I want the site navigation to expose the documented learning, reference, resource, and community areas so that I can reach the right implementation guidance.</x:v>
-      </x:c>
-      <x:c r="G481" s="13" t="str">
-        <x:v>Configured internal routes resolve, active navigation state is clear, expandable sections work, and external links open their intended destinations.</x:v>
-      </x:c>
-      <x:c r="H481" s="13" t="str">
-        <x:v>navigation.tabs; navigation.sections; navigation.expand; navigation.instant; nav entries</x:v>
-      </x:c>
-      <x:c r="I481" s="2" t="str">
-        <x:v>Needs fix</x:v>
-      </x:c>
-      <x:c r="J481" s="13" t="str">
-        <x:v>Generated-site sweep: 102 HTML pages loaded; 13 broken internal targets; 19 source pages are not in nav.</x:v>
-      </x:c>
-      <x:c r="K481" s="13" t="str">
-        <x:v>Live crawl found 9 internal target failures, including two source pages returning 404.</x:v>
-      </x:c>
-      <x:c r="L481" s="13" t="str">
-        <x:v>Repaired broken internal documentation targets and logged unlisted pages for navigation follow-up.</x:v>
-      </x:c>
-      <x:c r="M481" s="13" t="str">
-        <x:v>de9a6a7</x:v>
-      </x:c>
-      <x:c r="N481" s="13" t="str">
-        <x:v>Live recheck: 101 deployed pages crawled; 105 internal targets checked; 9 failed. Local fixes exist in de9a6a7, but the deployed site is stale.</x:v>
-      </x:c>
-      <x:c r="O481" s="25" t="str">
-        <x:v>Redeploy the committed documentation-link fixes, then rerun the live crawl.</x:v>
-      </x:c>
+      <x:c r="A481" s="16"/>
+      <x:c r="B481" s="2"/>
+      <x:c r="C481" s="2"/>
+      <x:c r="D481" s="2"/>
+      <x:c r="E481" s="2"/>
+      <x:c r="F481" s="13"/>
+      <x:c r="G481" s="13"/>
+      <x:c r="H481" s="13"/>
+      <x:c r="I481" s="2"/>
+      <x:c r="J481" s="13"/>
+      <x:c r="K481" s="13"/>
+      <x:c r="L481" s="13"/>
+      <x:c r="M481" s="13"/>
+      <x:c r="N481" s="13"/>
+      <x:c r="O481" s="25"/>
     </x:row>
     <x:row r="482" ht="42" customHeight="1">
-      <x:c r="A482" s="16" t="str">
-        <x:v>SITE-002</x:v>
-      </x:c>
-      <x:c r="B482" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C482" s="2" t="str">
-        <x:v>Search</x:v>
-      </x:c>
-      <x:c r="D482" s="2" t="str">
-        <x:v>Search</x:v>
-      </x:c>
-      <x:c r="E482" s="2" t="str">
-        <x:v>mkdocs.yml / Material search</x:v>
-      </x:c>
-      <x:c r="F482" s="13" t="str">
-        <x:v>As a developer, I want to search the docs by concept, symbol, or error text so that I can find implementation guidance without knowing the page location.</x:v>
-      </x:c>
-      <x:c r="G482" s="13" t="str">
-        <x:v>Search opens from the header, accepts text, highlights matches, and selecting a result lands on the matching page and section.</x:v>
-      </x:c>
-      <x:c r="H482" s="13" t="str">
-        <x:v>search.highlight; search.share; search.suggest</x:v>
-      </x:c>
-      <x:c r="I482" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J482" s="13" t="str">
-        <x:v>Browser: search for 'timelocks' returned 6 matching documents; selecting the first result opened Timelocks with an anchor.</x:v>
-      </x:c>
-      <x:c r="K482" s="13" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L482" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A482" s="16"/>
+      <x:c r="B482" s="2"/>
+      <x:c r="C482" s="2"/>
+      <x:c r="D482" s="2"/>
+      <x:c r="E482" s="2"/>
+      <x:c r="F482" s="13"/>
+      <x:c r="G482" s="13"/>
+      <x:c r="H482" s="13"/>
+      <x:c r="I482" s="2"/>
+      <x:c r="J482" s="13"/>
+      <x:c r="K482" s="13"/>
+      <x:c r="L482" s="13"/>
       <x:c r="M482" s="13"/>
-      <x:c r="N482" s="13" t="str">
-        <x:v>Browser search for `timelocks` returned 6 matching documents and share URL retained the query.</x:v>
-      </x:c>
-      <x:c r="O482" s="25" t="str">
-        <x:v>Test exact terms, no-result terms, and a result with an anchor.</x:v>
-      </x:c>
+      <x:c r="N482" s="13"/>
+      <x:c r="O482" s="25"/>
     </x:row>
     <x:row r="483" ht="42" customHeight="1">
-      <x:c r="A483" s="16" t="str">
-        <x:v>SITE-003</x:v>
-      </x:c>
-      <x:c r="B483" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C483" s="2" t="str">
-        <x:v>Theme toggle</x:v>
-      </x:c>
-      <x:c r="D483" s="2" t="str">
-        <x:v>Theme toggle</x:v>
-      </x:c>
-      <x:c r="E483" s="2" t="str">
-        <x:v>mkdocs.yml / docs/javascript/simplicity-embed.js</x:v>
-      </x:c>
-      <x:c r="F483" s="13" t="str">
-        <x:v>As a developer, I want to switch light and dark themes so that code and diagrams remain readable in my environment.</x:v>
-      </x:c>
-      <x:c r="G483" s="13" t="str">
-        <x:v>The theme toggle changes the host page without losing the current route, and embedded Try It content receives the same theme.</x:v>
-      </x:c>
-      <x:c r="H483" s="13" t="str">
-        <x:v>palette; data-md-color-scheme; simplicity-embed-set-theme</x:v>
-      </x:c>
-      <x:c r="I483" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J483" s="13" t="str">
-        <x:v>Browser: host dark theme selected, but embedded Try It URL remained theme=light and the frame rendered light.</x:v>
-      </x:c>
-      <x:c r="K483" s="13" t="str">
-        <x:v>Theme handoff is out of sync on the embedded page.</x:v>
-      </x:c>
-      <x:c r="L483" s="13" t="str">
-        <x:v>Synchronize embedded theme from the host palette.</x:v>
-      </x:c>
-      <x:c r="M483" s="13" t="str">
-        <x:v>f32c3fc</x:v>
-      </x:c>
-      <x:c r="N483" s="13" t="str">
-        <x:v>Host palette switched between light/default and dark/slate; iframe URL changed between `theme=light` and `theme=dark`.</x:v>
-      </x:c>
-      <x:c r="O483" s="25" t="str">
-        <x:v>Test light, dark, and system modes with and without an iframe.</x:v>
-      </x:c>
+      <x:c r="A483" s="16"/>
+      <x:c r="B483" s="2"/>
+      <x:c r="C483" s="2"/>
+      <x:c r="D483" s="2"/>
+      <x:c r="E483" s="2"/>
+      <x:c r="F483" s="13"/>
+      <x:c r="G483" s="13"/>
+      <x:c r="H483" s="13"/>
+      <x:c r="I483" s="2"/>
+      <x:c r="J483" s="13"/>
+      <x:c r="K483" s="13"/>
+      <x:c r="L483" s="13"/>
+      <x:c r="M483" s="13"/>
+      <x:c r="N483" s="13"/>
+      <x:c r="O483" s="25"/>
     </x:row>
     <x:row r="484" ht="42" customHeight="1">
-      <x:c r="A484" s="16" t="str">
-        <x:v>SITE-004</x:v>
-      </x:c>
-      <x:c r="B484" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C484" s="2" t="str">
-        <x:v>Instant navigation</x:v>
-      </x:c>
-      <x:c r="D484" s="2" t="str">
-        <x:v>Instant navigation</x:v>
-      </x:c>
-      <x:c r="E484" s="2" t="str">
-        <x:v>mkdocs.yml / Material navigation.instant</x:v>
-      </x:c>
-      <x:c r="F484" s="13" t="str">
-        <x:v>As a developer, I want internal navigation to preserve a fast browsing flow so that I can follow related concepts without a full reload.</x:v>
-      </x:c>
-      <x:c r="G484" s="13" t="str">
-        <x:v>Internal navigation swaps content, updates URL/title/active navigation, and re-wires embeds and MathJax on the new page.</x:v>
-      </x:c>
-      <x:c r="H484" s="13" t="str">
-        <x:v>navigation.instant; document$ subscriptions</x:v>
-      </x:c>
-      <x:c r="I484" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J484" s="13" t="str">
-        <x:v>Browser: search-result navigation changed route to /documentation/timelocks/?h=timelocks and refreshed page content.</x:v>
-      </x:c>
-      <x:c r="K484" s="13" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L484" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A484" s="16"/>
+      <x:c r="B484" s="2"/>
+      <x:c r="C484" s="2"/>
+      <x:c r="D484" s="2"/>
+      <x:c r="E484" s="2"/>
+      <x:c r="F484" s="13"/>
+      <x:c r="G484" s="13"/>
+      <x:c r="H484" s="13"/>
+      <x:c r="I484" s="2"/>
+      <x:c r="J484" s="13"/>
+      <x:c r="K484" s="13"/>
+      <x:c r="L484" s="13"/>
       <x:c r="M484" s="13"/>
-      <x:c r="N484" s="13" t="str">
-        <x:v>Search-result navigation reached `/documentation/timelocks/?h=timelocks` through the local site.</x:v>
-      </x:c>
-      <x:c r="O484" s="25" t="str">
-        <x:v>Navigate across a normal page, a glossary link, and an embedded page.</x:v>
-      </x:c>
+      <x:c r="N484" s="13"/>
+      <x:c r="O484" s="25"/>
     </x:row>
     <x:row r="485" ht="42" customHeight="1">
-      <x:c r="A485" s="16" t="str">
-        <x:v>SITE-005</x:v>
-      </x:c>
-      <x:c r="B485" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C485" s="2" t="str">
-        <x:v>Code actions</x:v>
-      </x:c>
-      <x:c r="D485" s="2" t="str">
-        <x:v>Code actions</x:v>
-      </x:c>
-      <x:c r="E485" s="2" t="str">
-        <x:v>mkdocs.yml</x:v>
-      </x:c>
-      <x:c r="F485" s="13" t="str">
-        <x:v>As a developer, I want to copy code and open the source of a page so that I can reproduce or inspect examples.</x:v>
-      </x:c>
-      <x:c r="G485" s="13" t="str">
-        <x:v>Code copy controls copy the intended block and source/edit controls point to the correct repository path when available.</x:v>
-      </x:c>
-      <x:c r="H485" s="13" t="str">
-        <x:v>content.code.copy; content.action.edit; overrides/partials/content.html</x:v>
-      </x:c>
-      <x:c r="I485" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J485" s="13" t="str">
-        <x:v>Browser AX tree exposed Edit this page and code copy/line-selection controls on rendered pages.</x:v>
-      </x:c>
-      <x:c r="K485" s="13" t="str">
-        <x:v>Copy action still needs a clipboard assertion.</x:v>
-      </x:c>
-      <x:c r="L485" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A485" s="16"/>
+      <x:c r="B485" s="2"/>
+      <x:c r="C485" s="2"/>
+      <x:c r="D485" s="2"/>
+      <x:c r="E485" s="2"/>
+      <x:c r="F485" s="13"/>
+      <x:c r="G485" s="13"/>
+      <x:c r="H485" s="13"/>
+      <x:c r="I485" s="2"/>
+      <x:c r="J485" s="13"/>
+      <x:c r="K485" s="13"/>
+      <x:c r="L485" s="13"/>
       <x:c r="M485" s="13"/>
-      <x:c r="N485" s="13" t="str">
-        <x:v>Rendered code blocks and Try It controls remained available; runnable example executed successfully.</x:v>
-      </x:c>
-      <x:c r="O485" s="25" t="str">
-        <x:v>Test a code-heavy page and a page with a generated title.</x:v>
-      </x:c>
+      <x:c r="N485" s="13"/>
+      <x:c r="O485" s="25"/>
     </x:row>
     <x:row r="486" ht="42" customHeight="1">
-      <x:c r="A486" s="16" t="str">
-        <x:v>SITE-006</x:v>
-      </x:c>
-      <x:c r="B486" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C486" s="2" t="str">
-        <x:v>Glossary previews</x:v>
-      </x:c>
-      <x:c r="D486" s="2" t="str">
-        <x:v>Glossary previews</x:v>
-      </x:c>
-      <x:c r="E486" s="2" t="str">
-        <x:v>includes/hooks/autolink_glossary.py / docs/glossary.md</x:v>
-      </x:c>
-      <x:c r="F486" s="13" t="str">
-        <x:v>As a developer, I want glossary links to preview definitions so that I can understand terminology without losing my place.</x:v>
-      </x:c>
-      <x:c r="G486" s="13" t="str">
-        <x:v>Glossary links receive the preview attribute, the preview content is readable, and ordinary links remain unchanged.</x:v>
-      </x:c>
-      <x:c r="H486" s="13" t="str">
-        <x:v>on_page_markdown regex; data-preview</x:v>
-      </x:c>
-      <x:c r="I486" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J486" s="13" t="str">
-        <x:v>Rendered HTML contains 809 data-preview attributes on glossary links.</x:v>
-      </x:c>
-      <x:c r="K486" s="13" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L486" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A486" s="16"/>
+      <x:c r="B486" s="2"/>
+      <x:c r="C486" s="2"/>
+      <x:c r="D486" s="2"/>
+      <x:c r="E486" s="2"/>
+      <x:c r="F486" s="13"/>
+      <x:c r="G486" s="13"/>
+      <x:c r="H486" s="13"/>
+      <x:c r="I486" s="2"/>
+      <x:c r="J486" s="13"/>
+      <x:c r="K486" s="13"/>
+      <x:c r="L486" s="13"/>
       <x:c r="M486" s="13"/>
-      <x:c r="N486" s="13" t="str">
-        <x:v>Generated HTML retained 809 glossary-preview attributes across 102 HTML pages.</x:v>
-      </x:c>
-      <x:c r="O486" s="25" t="str">
-        <x:v>Build and inspect glossary links across representative pages.</x:v>
-      </x:c>
+      <x:c r="N486" s="13"/>
+      <x:c r="O486" s="25"/>
     </x:row>
     <x:row r="487" ht="42" customHeight="1">
-      <x:c r="A487" s="16" t="str">
-        <x:v>SITE-007</x:v>
-      </x:c>
-      <x:c r="B487" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C487" s="2" t="str">
-        <x:v>Math rendering</x:v>
-      </x:c>
-      <x:c r="D487" s="2" t="str">
-        <x:v>Math rendering</x:v>
-      </x:c>
-      <x:c r="E487" s="2" t="str">
-        <x:v>docs/javascript/mathjax.js / mkdocs.yml</x:v>
-      </x:c>
-      <x:c r="F487" s="13" t="str">
-        <x:v>As a developer, I want inline and display math to render correctly so that formal definitions and equations are usable.</x:v>
-      </x:c>
-      <x:c r="G487" s="13" t="str">
-        <x:v>Configured delimiters render after initial load and after instant-navigation page swaps, without leaving raw delimiters or console errors.</x:v>
-      </x:c>
-      <x:c r="H487" s="13" t="str">
-        <x:v>MathJax tex delimiters; document.subscribe</x:v>
-      </x:c>
-      <x:c r="I487" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J487" s="13" t="str">
-        <x:v>All 100 generated page shells include mathjax.js; post-navigation typesetting still needs a math-bearing page assertion.</x:v>
-      </x:c>
-      <x:c r="K487" s="13" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L487" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A487" s="16"/>
+      <x:c r="B487" s="2"/>
+      <x:c r="C487" s="2"/>
+      <x:c r="D487" s="2"/>
+      <x:c r="E487" s="2"/>
+      <x:c r="F487" s="13"/>
+      <x:c r="G487" s="13"/>
+      <x:c r="H487" s="13"/>
+      <x:c r="I487" s="2"/>
+      <x:c r="J487" s="13"/>
+      <x:c r="K487" s="13"/>
+      <x:c r="L487" s="13"/>
       <x:c r="M487" s="13"/>
-      <x:c r="N487" s="13" t="str">
-        <x:v>Generated page shells loaded with headings; MathJax assets were present in the built site.</x:v>
-      </x:c>
-      <x:c r="O487" s="25" t="str">
-        <x:v>Test a page with inline and display math and navigate away and back.</x:v>
-      </x:c>
+      <x:c r="N487" s="13"/>
+      <x:c r="O487" s="25"/>
     </x:row>
     <x:row r="488" ht="42" customHeight="1">
-      <x:c r="A488" s="16" t="str">
-        <x:v>SITE-008</x:v>
-      </x:c>
-      <x:c r="B488" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C488" s="2" t="str">
-        <x:v>Embedded Try It frame</x:v>
-      </x:c>
-      <x:c r="D488" s="2" t="str">
-        <x:v>Embedded Try It frame</x:v>
-      </x:c>
-      <x:c r="E488" s="2" t="str">
-        <x:v>docs/javascript/simplicity-embed.js / docs/getting-started/try-it.md</x:v>
-      </x:c>
-      <x:c r="F488" s="13" t="str">
-        <x:v>As a developer, I want the embedded Try It experience to load inside the documentation so that I can try examples without leaving the learning flow.</x:v>
-      </x:c>
-      <x:c r="G488" s="13" t="str">
-        <x:v>The iframe gets embed and theme parameters, fills the available width, and resizes to messages from its own content window.</x:v>
-      </x:c>
-      <x:c r="H488" s="13" t="str">
-        <x:v>iframe.simplicity-embed; data-tut-src; simplicity-embed-resize</x:v>
-      </x:c>
-      <x:c r="I488" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J488" s="13" t="str">
-        <x:v>Browser: iframe loaded with embed=1, but theme parameter did not match the dark host during instant navigation.</x:v>
-      </x:c>
-      <x:c r="K488" s="13" t="str">
-        <x:v>Fix theme propagation together with SITE-003.</x:v>
-      </x:c>
-      <x:c r="L488" s="13" t="str">
-        <x:v>Synchronize embedded theme from the host palette after navigation and palette changes.</x:v>
-      </x:c>
-      <x:c r="M488" s="13" t="str">
-        <x:v>f32c3fc</x:v>
-      </x:c>
-      <x:c r="N488" s="13" t="str">
-        <x:v>Try It iframe followed host palette: `theme=dark` under slate and `theme=light` under default.</x:v>
-      </x:c>
-      <x:c r="O488" s="25" t="str">
-        <x:v>Test first load, instant navigation, resize, and theme changes.</x:v>
-      </x:c>
+      <x:c r="A488" s="16"/>
+      <x:c r="B488" s="2"/>
+      <x:c r="C488" s="2"/>
+      <x:c r="D488" s="2"/>
+      <x:c r="E488" s="2"/>
+      <x:c r="F488" s="13"/>
+      <x:c r="G488" s="13"/>
+      <x:c r="H488" s="13"/>
+      <x:c r="I488" s="2"/>
+      <x:c r="J488" s="13"/>
+      <x:c r="K488" s="13"/>
+      <x:c r="L488" s="13"/>
+      <x:c r="M488" s="13"/>
+      <x:c r="N488" s="13"/>
+      <x:c r="O488" s="25"/>
     </x:row>
     <x:row r="489" ht="42" customHeight="1">
-      <x:c r="A489" s="16" t="str">
-        <x:v>SITE-009</x:v>
-      </x:c>
-      <x:c r="B489" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C489" s="2" t="str">
-        <x:v>404 recovery</x:v>
-      </x:c>
-      <x:c r="D489" s="2" t="str">
-        <x:v>404 recovery</x:v>
-      </x:c>
-      <x:c r="E489" s="2" t="str">
-        <x:v>overrides/404.html</x:v>
-      </x:c>
-      <x:c r="F489" s="13" t="str">
-        <x:v>As a developer, I want a missing page to offer recovery actions so that a broken link does not end my documentation task.</x:v>
-      </x:c>
-      <x:c r="G489" s="13" t="str">
-        <x:v>The 404 page identifies the error, returns home, opens documentation search, and provides a broken-link report with the current URL.</x:v>
-      </x:c>
-      <x:c r="H489" s="13" t="str">
-        <x:v>overrides/404.html</x:v>
-      </x:c>
-      <x:c r="I489" s="2" t="str">
-        <x:v>Needs fix</x:v>
-      </x:c>
-      <x:c r="J489" s="13" t="str">
-        <x:v>Browser: 404 page rendered and search/home recovery worked, but GitHub report href contained body '404 Error at URL: /' instead of /missing-page/.</x:v>
-      </x:c>
-      <x:c r="K489" s="13" t="str">
-        <x:v>Live 404 report still hard-codes `/.` instead of the missing browser URL.</x:v>
-      </x:c>
-      <x:c r="L489" s="13" t="str">
-        <x:v>Build the broken-link report body from the current browser URL.</x:v>
-      </x:c>
-      <x:c r="M489" s="13" t="str">
-        <x:v>2617714</x:v>
-      </x:c>
-      <x:c r="N489" s="13" t="str">
-        <x:v>Live recheck at `/live-audit-missing-page/`: report body was `404 Error at URL: /.`. Local fix exists in 2617714, but it is not deployed.</x:v>
-      </x:c>
-      <x:c r="O489" s="25" t="str">
-        <x:v>Redeploy the 404 template fix, then verify the report body includes the actual missing path.</x:v>
-      </x:c>
+      <x:c r="A489" s="16"/>
+      <x:c r="B489" s="2"/>
+      <x:c r="C489" s="2"/>
+      <x:c r="D489" s="2"/>
+      <x:c r="E489" s="2"/>
+      <x:c r="F489" s="13"/>
+      <x:c r="G489" s="13"/>
+      <x:c r="H489" s="13"/>
+      <x:c r="I489" s="2"/>
+      <x:c r="J489" s="13"/>
+      <x:c r="K489" s="13"/>
+      <x:c r="L489" s="13"/>
+      <x:c r="M489" s="13"/>
+      <x:c r="N489" s="13"/>
+      <x:c r="O489" s="25"/>
     </x:row>
     <x:row r="490" ht="42" customHeight="1">
-      <x:c r="A490" s="16" t="str">
-        <x:v>SITE-010</x:v>
-      </x:c>
-      <x:c r="B490" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C490" s="2" t="str">
-        <x:v>Page feedback</x:v>
-      </x:c>
-      <x:c r="D490" s="2" t="str">
-        <x:v>Page feedback</x:v>
-      </x:c>
-      <x:c r="E490" s="2" t="str">
-        <x:v>mkdocs.yml / Material feedback</x:v>
-      </x:c>
-      <x:c r="F490" s="13" t="str">
-        <x:v>As a developer, I want to report whether a page helped so that documentation gaps can be surfaced to maintainers.</x:v>
-      </x:c>
-      <x:c r="G490" s="13" t="str">
-        <x:v>Helpful and not-helpful choices are visible, acknowledge the selection, and the improvement path opens a correctly labeled issue form.</x:v>
-      </x:c>
-      <x:c r="H490" s="13" t="str">
-        <x:v>extra.analytics.feedback; content feedback partial</x:v>
-      </x:c>
-      <x:c r="I490" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J490" s="13" t="str">
-        <x:v>Browser: clicking 'This page was helpful' disabled the feedback control and displayed 'Thanks for your feedback!'.</x:v>
-      </x:c>
-      <x:c r="K490" s="13" t="str">
-        <x:v>Negative path and issue-form link still need assertion.</x:v>
-      </x:c>
-      <x:c r="L490" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A490" s="16"/>
+      <x:c r="B490" s="2"/>
+      <x:c r="C490" s="2"/>
+      <x:c r="D490" s="2"/>
+      <x:c r="E490" s="2"/>
+      <x:c r="F490" s="13"/>
+      <x:c r="G490" s="13"/>
+      <x:c r="H490" s="13"/>
+      <x:c r="I490" s="2"/>
+      <x:c r="J490" s="13"/>
+      <x:c r="K490" s="13"/>
+      <x:c r="L490" s="13"/>
       <x:c r="M490" s="13"/>
-      <x:c r="N490" s="13" t="str">
-        <x:v>Helpful feedback produced `Thanks for your feedback!` and disabled both feedback controls.</x:v>
-      </x:c>
-      <x:c r="O490" s="25" t="str">
-        <x:v>Test both ratings and the generated issue link.</x:v>
-      </x:c>
+      <x:c r="N490" s="13"/>
+      <x:c r="O490" s="25"/>
     </x:row>
     <x:row r="491" ht="42" customHeight="1">
-      <x:c r="A491" s="16" t="str">
-        <x:v>SITE-011</x:v>
-      </x:c>
-      <x:c r="B491" s="2" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C491" s="2" t="str">
-        <x:v>Homepage conversion paths</x:v>
-      </x:c>
-      <x:c r="D491" s="2" t="str">
-        <x:v>Homepage conversion paths</x:v>
-      </x:c>
-      <x:c r="E491" s="2" t="str">
-        <x:v>overrides/main.html / docs/index.md</x:v>
-      </x:c>
-      <x:c r="F491" s="13" t="str">
-        <x:v>As a new developer, I want the homepage to offer clear paths into the quickstart, reference, and browser Try It experience so that I can start building quickly.</x:v>
-      </x:c>
-      <x:c r="G491" s="13" t="str">
-        <x:v>The hero renders once, its buttons target valid routes, the main examples remain readable, and the live-on-Liquid status links to the relevant announcement.</x:v>
-      </x:c>
-      <x:c r="H491" s="13" t="str">
-        <x:v>hero; Get Started; Read the Docs; Try it in Your Browser</x:v>
-      </x:c>
-      <x:c r="I491" s="2" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J491" s="13" t="str">
-        <x:v>Browser AX tree exposed hero links for Get Started, Read the Docs, Try it in Your Browser, and the Liquid mainnet announcement.</x:v>
-      </x:c>
-      <x:c r="K491" s="13" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L491" s="13" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A491" s="16"/>
+      <x:c r="B491" s="2"/>
+      <x:c r="C491" s="2"/>
+      <x:c r="D491" s="2"/>
+      <x:c r="E491" s="2"/>
+      <x:c r="F491" s="13"/>
+      <x:c r="G491" s="13"/>
+      <x:c r="H491" s="13"/>
+      <x:c r="I491" s="2"/>
+      <x:c r="J491" s="13"/>
+      <x:c r="K491" s="13"/>
+      <x:c r="L491" s="13"/>
       <x:c r="M491" s="13"/>
-      <x:c r="N491" s="13" t="str">
-        <x:v>Homepage and navigation route checks returned HTTP 200 with headings.</x:v>
-      </x:c>
-      <x:c r="O491" s="25" t="str">
-        <x:v>Test each hero link in light and dark themes.</x:v>
-      </x:c>
+      <x:c r="N491" s="13"/>
+      <x:c r="O491" s="25"/>
     </x:row>
     <x:row r="492" ht="42" customHeight="1">
-      <x:c r="A492" s="20" t="str">
-        <x:v>TRY-001</x:v>
-      </x:c>
-      <x:c r="B492" s="26" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C492" s="26" t="str">
-        <x:v>Try It app load</x:v>
-      </x:c>
-      <x:c r="D492" s="26" t="str">
-        <x:v>Try It app load</x:v>
-      </x:c>
-      <x:c r="E492" s="26" t="str">
-        <x:v>docs/getting-started/try-it/try/index.html</x:v>
-      </x:c>
-      <x:c r="F492" s="27" t="str">
-        <x:v>As a developer, I want the Try It app to load its tutorial and editor so that I can experiment with SimplicityHL in the browser.</x:v>
-      </x:c>
-      <x:c r="G492" s="27" t="str">
-        <x:v>The static app loads its scripts and WASM, shows tutorial content and an editor, and does not fail due to missing assets.</x:v>
-      </x:c>
-      <x:c r="H492" s="27" t="str">
-        <x:v>Astro bundle; simptut_wasm; runnable bundle</x:v>
-      </x:c>
-      <x:c r="I492" s="26" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J492" s="27" t="str">
-        <x:v>Browser: embedded Try It app loaded its WASM-backed lesson content and editor.</x:v>
-      </x:c>
-      <x:c r="K492" s="27" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L492" s="27" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A492" s="20"/>
+      <x:c r="B492" s="26"/>
+      <x:c r="C492" s="26"/>
+      <x:c r="D492" s="26"/>
+      <x:c r="E492" s="26"/>
+      <x:c r="F492" s="27"/>
+      <x:c r="G492" s="27"/>
+      <x:c r="H492" s="27"/>
+      <x:c r="I492" s="26"/>
+      <x:c r="J492" s="27"/>
+      <x:c r="K492" s="27"/>
+      <x:c r="L492" s="27"/>
       <x:c r="M492" s="27"/>
-      <x:c r="N492" s="27" t="str">
-        <x:v>Try It page loaded with embedded compiler content and three Run controls.</x:v>
-      </x:c>
-      <x:c r="O492" s="28" t="str">
-        <x:v>Load the bundled app directly and through the docs iframe.</x:v>
-      </x:c>
+      <x:c r="N492" s="27"/>
+      <x:c r="O492" s="28"/>
     </x:row>
     <x:row r="493" ht="42" customHeight="1">
-      <x:c r="A493" t="str">
-        <x:v>TRY-002</x:v>
-      </x:c>
-      <x:c r="B493" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C493" t="str">
-        <x:v>Try It tutorial navigation</x:v>
-      </x:c>
-      <x:c r="D493" t="str">
-        <x:v>Try It tutorial navigation</x:v>
-      </x:c>
-      <x:c r="E493" t="str">
-        <x:v>docs/getting-started/try-it/_astro/page.Dwipeu-R.js / index.html</x:v>
-      </x:c>
-      <x:c r="F493" s="29" t="str">
-        <x:v>As a developer, I want to move between tutorial sections so that I can learn the language in sequence.</x:v>
-      </x:c>
-      <x:c r="G493" s="29" t="str">
-        <x:v>Tutorial navigation, table of contents, and mobile navigation change the visible lesson without broken links or stale selection.</x:v>
-      </x:c>
-      <x:c r="H493" s="29" t="str">
-        <x:v>starlight-toc; TableOfContents; MobileTableOfContents</x:v>
-      </x:c>
-      <x:c r="I493" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J493" s="29" t="str">
-        <x:v>Browser AX tree exposed the Try It table of contents and lesson headings.</x:v>
-      </x:c>
-      <x:c r="K493" s="29" t="str">
-        <x:v>Narrow viewport/mobile navigation still needs assertion.</x:v>
-      </x:c>
-      <x:c r="L493" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A493"/>
+      <x:c r="B493"/>
+      <x:c r="C493"/>
+      <x:c r="D493"/>
+      <x:c r="E493"/>
+      <x:c r="F493" s="29"/>
+      <x:c r="G493" s="29"/>
+      <x:c r="H493" s="29"/>
+      <x:c r="I493"/>
+      <x:c r="J493" s="29"/>
+      <x:c r="K493" s="29"/>
+      <x:c r="L493" s="29"/>
       <x:c r="M493" s="29"/>
-      <x:c r="N493" s="29" t="str">
-        <x:v>Embedded tutorial headings and next-step links were present.</x:v>
-      </x:c>
-      <x:c r="O493" s="29" t="str">
-        <x:v>Test desktop and narrow viewport navigation.</x:v>
-      </x:c>
+      <x:c r="N493" s="29"/>
+      <x:c r="O493" s="29"/>
     </x:row>
     <x:row r="494" ht="42" customHeight="1">
-      <x:c r="A494" t="str">
-        <x:v>TRY-003</x:v>
-      </x:c>
-      <x:c r="B494" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C494" t="str">
-        <x:v>Try It runnable examples</x:v>
-      </x:c>
-      <x:c r="D494" t="str">
-        <x:v>Try It runnable examples</x:v>
-      </x:c>
-      <x:c r="E494" t="str">
-        <x:v>docs/getting-started/try-it/_astro/runnable.Bqd5ptkk.js</x:v>
-      </x:c>
-      <x:c r="F494" s="29" t="str">
-        <x:v>As a developer, I want to run the example code so that I can see whether the lesson behaves as described.</x:v>
-      </x:c>
-      <x:c r="G494" s="29" t="str">
-        <x:v>Runnable controls execute the selected example, show output or a useful error, and keep the page responsive while WASM runs.</x:v>
-      </x:c>
-      <x:c r="H494" s="29" t="str">
-        <x:v>runnable bundle; simptut_wasm.js</x:v>
-      </x:c>
-      <x:c r="I494" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J494" s="29" t="str">
-        <x:v>Browser: first runnable example returned 'Program succeeded — all assertions held' with a CMR.</x:v>
-      </x:c>
-      <x:c r="K494" s="29" t="str">
-        <x:v>Invalid assertion path was not editable through the current accessibility target.</x:v>
-      </x:c>
-      <x:c r="L494" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A494"/>
+      <x:c r="B494"/>
+      <x:c r="C494"/>
+      <x:c r="D494"/>
+      <x:c r="E494"/>
+      <x:c r="F494" s="29"/>
+      <x:c r="G494" s="29"/>
+      <x:c r="H494" s="29"/>
+      <x:c r="I494"/>
+      <x:c r="J494" s="29"/>
+      <x:c r="K494" s="29"/>
+      <x:c r="L494" s="29"/>
       <x:c r="M494" s="29"/>
-      <x:c r="N494" s="29" t="str">
-        <x:v>First Try It example ran and displayed `Program succeeded — all assertions held` with a CMR.</x:v>
-      </x:c>
-      <x:c r="O494" s="29" t="str">
-        <x:v>Run a valid example and an invalid edit if the UI exposes editing.</x:v>
-      </x:c>
+      <x:c r="N494" s="29"/>
+      <x:c r="O494" s="29"/>
     </x:row>
     <x:row r="495" ht="42" customHeight="1">
-      <x:c r="A495" t="str">
-        <x:v>TRY-004</x:v>
-      </x:c>
-      <x:c r="B495" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C495" t="str">
-        <x:v>Try It search</x:v>
-      </x:c>
-      <x:c r="D495" t="str">
-        <x:v>Try It search</x:v>
-      </x:c>
-      <x:c r="E495" t="str">
-        <x:v>docs/getting-started/try-it/pagefind/</x:v>
-      </x:c>
-      <x:c r="F495" s="29" t="str">
-        <x:v>As a developer, I want to search the Try It documentation so that I can find a lesson or symbol quickly.</x:v>
-      </x:c>
-      <x:c r="G495" s="29" t="str">
-        <x:v>Search opens, accepts a query, returns relevant results, and selecting a result updates the app route.</x:v>
-      </x:c>
-      <x:c r="H495" s="29" t="str">
-        <x:v>pagefind UI and index assets</x:v>
-      </x:c>
-      <x:c r="I495" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J495" s="29" t="str">
-        <x:v>Static bundle contains Pagefind UI, worker, index, and fragment assets.</x:v>
-      </x:c>
-      <x:c r="K495" s="29" t="str">
-        <x:v>Browser search interaction still needs assertion.</x:v>
-      </x:c>
-      <x:c r="L495" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A495"/>
+      <x:c r="B495"/>
+      <x:c r="C495"/>
+      <x:c r="D495"/>
+      <x:c r="E495"/>
+      <x:c r="F495" s="29"/>
+      <x:c r="G495" s="29"/>
+      <x:c r="H495" s="29"/>
+      <x:c r="I495"/>
+      <x:c r="J495" s="29"/>
+      <x:c r="K495" s="29"/>
+      <x:c r="L495" s="29"/>
       <x:c r="M495" s="29"/>
-      <x:c r="N495" s="29" t="str">
-        <x:v>Try It search control returned matching documents through the bundled Pagefind index.</x:v>
-      </x:c>
-      <x:c r="O495" s="29" t="str">
-        <x:v>Test a known tutorial term and a no-result term.</x:v>
-      </x:c>
+      <x:c r="N495" s="29"/>
+      <x:c r="O495" s="29"/>
     </x:row>
     <x:row r="496" ht="42" customHeight="1">
-      <x:c r="A496" t="str">
-        <x:v>TRY-005</x:v>
-      </x:c>
-      <x:c r="B496" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C496" t="str">
-        <x:v>Try It print and 404</x:v>
-      </x:c>
-      <x:c r="D496" t="str">
-        <x:v>Try It print and 404</x:v>
-      </x:c>
-      <x:c r="E496" t="str">
-        <x:v>docs/getting-started/try-it/_astro/print.ehPL0gv-.css / 404.html</x:v>
-      </x:c>
-      <x:c r="F496" s="29" t="str">
-        <x:v>As a developer, I want the Try It app to print or recover from a missing lesson so that the experience remains usable outside the happy path.</x:v>
-      </x:c>
-      <x:c r="G496" s="29" t="str">
-        <x:v>Print styles hide interactive chrome appropriately, and missing app routes show a recoverable 404 page.</x:v>
-      </x:c>
-      <x:c r="H496" s="29" t="str">
-        <x:v>print stylesheet; app 404.html</x:v>
-      </x:c>
-      <x:c r="I496" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J496" s="29" t="str">
-        <x:v>Static bundle contains print CSS and app 404.html; direct missing route is handled by the outer docs 404.</x:v>
-      </x:c>
-      <x:c r="K496" s="29" t="str">
-        <x:v>Print preview needs assertion.</x:v>
-      </x:c>
-      <x:c r="L496" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A496"/>
+      <x:c r="B496"/>
+      <x:c r="C496"/>
+      <x:c r="D496"/>
+      <x:c r="E496"/>
+      <x:c r="F496" s="29"/>
+      <x:c r="G496" s="29"/>
+      <x:c r="H496" s="29"/>
+      <x:c r="I496"/>
+      <x:c r="J496" s="29"/>
+      <x:c r="K496" s="29"/>
+      <x:c r="L496" s="29"/>
       <x:c r="M496" s="29"/>
-      <x:c r="N496" s="29" t="str">
-        <x:v>Try It route and generated 404 support assets were present in the local build; external print output not exercised.</x:v>
-      </x:c>
-      <x:c r="O496" s="29" t="str">
-        <x:v>Use print preview and request a nonexistent nested route.</x:v>
-      </x:c>
+      <x:c r="N496" s="29"/>
+      <x:c r="O496" s="29"/>
     </x:row>
     <x:row r="497" ht="42" customHeight="1">
-      <x:c r="A497" t="str">
-        <x:v>SITE-012</x:v>
-      </x:c>
-      <x:c r="B497" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C497" t="str">
-        <x:v>Build hook</x:v>
-      </x:c>
-      <x:c r="D497" t="str">
-        <x:v>Build hygiene</x:v>
-      </x:c>
-      <x:c r="E497" t="str">
-        <x:v>includes/hooks/autolink_glossary.py</x:v>
-      </x:c>
-      <x:c r="F497" s="29" t="str">
-        <x:v>As a maintainer, I want the Markdown hook to transform content without unrelated filesystem side effects so that builds remain reproducible.</x:v>
-      </x:c>
-      <x:c r="G497" s="29" t="str">
-        <x:v>The hook only applies the intended glossary-link transformation and does not create arbitrary temp files.</x:v>
-      </x:c>
-      <x:c r="H497" s="29" t="str">
-        <x:v>on_page_markdown; current /tmp/foobaz write</x:v>
-      </x:c>
-      <x:c r="I497" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J497" s="29" t="str">
-        <x:v>Strict build created /tmp/foobaz.</x:v>
-      </x:c>
-      <x:c r="K497" s="29" t="str">
-        <x:v>Remove the unrelated write.</x:v>
-      </x:c>
-      <x:c r="L497" s="29" t="str">
-        <x:v>Remove the build hook's temporary `/tmp/foobaz` write.</x:v>
-      </x:c>
-      <x:c r="M497" s="29" t="str">
-        <x:v>33f6bcd</x:v>
-      </x:c>
-      <x:c r="N497" s="29" t="str">
-        <x:v>Clean build exited 0 and did not recreate `/tmp/foobaz`.</x:v>
-      </x:c>
+      <x:c r="A497"/>
+      <x:c r="B497"/>
+      <x:c r="C497"/>
+      <x:c r="D497"/>
+      <x:c r="E497"/>
+      <x:c r="F497" s="29"/>
+      <x:c r="G497" s="29"/>
+      <x:c r="H497" s="29"/>
+      <x:c r="I497"/>
+      <x:c r="J497" s="29"/>
+      <x:c r="K497" s="29"/>
+      <x:c r="L497" s="29"/>
+      <x:c r="M497" s="29"/>
+      <x:c r="N497" s="29"/>
       <x:c r="O497" s="29"/>
     </x:row>
     <x:row r="498" ht="42" customHeight="1">
-      <x:c r="A498" t="str">
-        <x:v>SITE-013</x:v>
-      </x:c>
-      <x:c r="B498" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C498" t="str">
-        <x:v>LLM exports</x:v>
-      </x:c>
-      <x:c r="D498" t="str">
-        <x:v>Machine-readable docs</x:v>
-      </x:c>
-      <x:c r="E498" t="str">
-        <x:v>mkdocs.yml / llms-source plugin</x:v>
-      </x:c>
-      <x:c r="F498" s="29" t="str">
-        <x:v>As an AI-assisted developer, I want machine-readable site exports so that I can discover and use the documentation programmatically.</x:v>
-      </x:c>
-      <x:c r="G498" s="29" t="str">
-        <x:v>The build publishes llms.txt and llms-full.txt with current page content and valid links.</x:v>
-      </x:c>
-      <x:c r="H498" s="29" t="str">
-        <x:v>llms-source output</x:v>
-      </x:c>
-      <x:c r="I498" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J498" s="29" t="str">
-        <x:v>Strict build generated both files.</x:v>
-      </x:c>
-      <x:c r="K498" s="29" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L498" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A498"/>
+      <x:c r="B498"/>
+      <x:c r="C498"/>
+      <x:c r="D498"/>
+      <x:c r="E498"/>
+      <x:c r="F498" s="29"/>
+      <x:c r="G498" s="29"/>
+      <x:c r="H498" s="29"/>
+      <x:c r="I498"/>
+      <x:c r="J498" s="29"/>
+      <x:c r="K498" s="29"/>
+      <x:c r="L498" s="29"/>
       <x:c r="M498" s="29"/>
-      <x:c r="N498" s="29" t="str">
-        <x:v>Build generated `site/llms.txt` and `site/llms-full.txt` and copied 99 Markdown files.</x:v>
-      </x:c>
+      <x:c r="N498" s="29"/>
       <x:c r="O498" s="29"/>
     </x:row>
     <x:row r="499" ht="42" customHeight="1">
-      <x:c r="A499" t="str">
-        <x:v>SITE-014</x:v>
-      </x:c>
-      <x:c r="B499" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C499" t="str">
-        <x:v>Revision metadata</x:v>
-      </x:c>
-      <x:c r="D499" t="str">
-        <x:v>Trust and provenance</x:v>
-      </x:c>
-      <x:c r="E499" t="str">
-        <x:v>mkdocs.yml / git-revision-date-localized / git-committers</x:v>
-      </x:c>
-      <x:c r="F499" s="29" t="str">
-        <x:v>As a developer, I want page revision and contributor information so that I can judge whether guidance is current and find maintainers.</x:v>
-      </x:c>
-      <x:c r="G499" s="29" t="str">
-        <x:v>Rendered pages show the configured date and contributor metadata without blocking builds when the API is unavailable.</x:v>
-      </x:c>
-      <x:c r="H499" s="29" t="str">
-        <x:v>git plugin output</x:v>
-      </x:c>
-      <x:c r="I499" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J499" s="29" t="str">
-        <x:v>Rendered page showed date and GitHub contributors.</x:v>
-      </x:c>
-      <x:c r="K499" s="29" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L499" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A499"/>
+      <x:c r="B499"/>
+      <x:c r="C499"/>
+      <x:c r="D499"/>
+      <x:c r="E499"/>
+      <x:c r="F499" s="29"/>
+      <x:c r="G499" s="29"/>
+      <x:c r="H499" s="29"/>
+      <x:c r="I499"/>
+      <x:c r="J499" s="29"/>
+      <x:c r="K499" s="29"/>
+      <x:c r="L499" s="29"/>
       <x:c r="M499" s="29"/>
-      <x:c r="N499" s="29" t="str">
-        <x:v>Built pages retained revision metadata/author blocks where configured.</x:v>
-      </x:c>
+      <x:c r="N499" s="29"/>
       <x:c r="O499" s="29"/>
     </x:row>
     <x:row r="500" ht="42" customHeight="1">
-      <x:c r="A500" t="str">
-        <x:v>SITE-015</x:v>
-      </x:c>
-      <x:c r="B500" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C500" t="str">
-        <x:v>Announcement dismissal</x:v>
-      </x:c>
-      <x:c r="D500" t="str">
-        <x:v>Navigation</x:v>
-      </x:c>
-      <x:c r="E500" t="str">
-        <x:v>mkdocs.yml / announce.dismiss</x:v>
-      </x:c>
-      <x:c r="F500" s="29" t="str">
-        <x:v>As a returning developer, I want to dismiss an announcement so that it does not obstruct reading on later visits.</x:v>
-      </x:c>
-      <x:c r="G500" s="29" t="str">
-        <x:v>The announcement dismiss control is visible when an announcement exists and persists its dismissal locally.</x:v>
-      </x:c>
-      <x:c r="H500" s="29" t="str">
-        <x:v>announce.dismiss</x:v>
-      </x:c>
-      <x:c r="I500" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J500" s="29" t="str">
-        <x:v>Configured but not browser-asserted.</x:v>
-      </x:c>
-      <x:c r="K500" s="29" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L500" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A500"/>
+      <x:c r="B500"/>
+      <x:c r="C500"/>
+      <x:c r="D500"/>
+      <x:c r="E500"/>
+      <x:c r="F500" s="29"/>
+      <x:c r="G500" s="29"/>
+      <x:c r="H500" s="29"/>
+      <x:c r="I500"/>
+      <x:c r="J500" s="29"/>
+      <x:c r="K500" s="29"/>
+      <x:c r="L500" s="29"/>
       <x:c r="M500" s="29"/>
-      <x:c r="N500" s="29" t="str">
-        <x:v>Built page chrome rendered without console-visible build failures in the tested flows.</x:v>
-      </x:c>
+      <x:c r="N500" s="29"/>
       <x:c r="O500" s="29"/>
     </x:row>
     <x:row r="501" ht="42" customHeight="1">
-      <x:c r="A501" t="str">
-        <x:v>SITE-016</x:v>
-      </x:c>
-      <x:c r="B501" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C501" t="str">
-        <x:v>Keyboard and page navigation</x:v>
-      </x:c>
-      <x:c r="D501" t="str">
-        <x:v>Accessibility</x:v>
-      </x:c>
-      <x:c r="E501" t="str">
-        <x:v>mkdocs.yml / Material theme</x:v>
-      </x:c>
-      <x:c r="F501" s="29" t="str">
-        <x:v>As a developer navigating by keyboard or a long page, I want skip-to-content and Back to top controls so that I can move efficiently.</x:v>
-      </x:c>
-      <x:c r="G501" s="29" t="str">
-        <x:v>The controls are present, focusable, and move focus or scroll to the intended destination.</x:v>
-      </x:c>
-      <x:c r="H501" s="29" t="str">
-        <x:v>skip-to-content; Back to top</x:v>
-      </x:c>
-      <x:c r="I501" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="J501" s="29" t="str">
-        <x:v>AX tree exposed both controls.</x:v>
-      </x:c>
-      <x:c r="K501" s="29" t="str">
-        <x:v>Baseline issue resolved or behavior verified.</x:v>
-      </x:c>
-      <x:c r="L501" s="29" t="str">
-        <x:v>No code change required.</x:v>
-      </x:c>
+      <x:c r="A501"/>
+      <x:c r="B501"/>
+      <x:c r="C501"/>
+      <x:c r="D501"/>
+      <x:c r="E501"/>
+      <x:c r="F501" s="29"/>
+      <x:c r="G501" s="29"/>
+      <x:c r="H501" s="29"/>
+      <x:c r="I501"/>
+      <x:c r="J501" s="29"/>
+      <x:c r="K501" s="29"/>
+      <x:c r="L501" s="29"/>
       <x:c r="M501" s="29"/>
-      <x:c r="N501" s="29" t="str">
-        <x:v>Accessibility tree exposed keyboard-settable search/theme controls and Back to top.</x:v>
-      </x:c>
+      <x:c r="N501" s="29"/>
       <x:c r="O501" s="29"/>
     </x:row>
   </x:sheetData>
@@ -21229,7 +20597,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98500487f13b4318"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4a64279d2944f3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>